<commit_message>
corrected remaining errors in witness files and in meta files
</commit_message>
<xml_diff>
--- a/data/meta/Witness_list_sheet.xlsx
+++ b/data/meta/Witness_list_sheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rkjin\github\Sirah-Project\data\meta\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{215AEE24-1E38-4B65-BEB6-E01074C7D063}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70504173-9427-4472-9CD7-B0986782F42A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="618" uniqueCount="518">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="624" uniqueCount="522">
   <si>
     <t>Arabic name</t>
   </si>
@@ -4245,6 +4245,18 @@
   </si>
   <si>
     <t>8/05/26 tagged and formatted, not in github as of this date.</t>
+  </si>
+  <si>
+    <t>WHZZY</t>
+  </si>
+  <si>
+    <t>حماد بن زيد الهمداني الخارقي الكوفي</t>
+  </si>
+  <si>
+    <t>Ḥammād b. Zayd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8/05/26 Name added to directory. Not added to github as of this date. </t>
   </si>
 </sst>
 </file>
@@ -4407,7 +4419,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -4433,14 +4445,28 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
@@ -4450,19 +4476,14 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4679,7 +4700,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AA1001"/>
+  <dimension ref="A1:AA1002"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.140625" customWidth="1"/>
@@ -4694,35 +4715,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A1" s="15"/>
-      <c r="B1" s="9" t="s">
+      <c r="A1" s="21"/>
+      <c r="B1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="E1" s="12" t="s">
         <v>3</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="14" t="s">
+      <c r="G1" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="14" t="s">
+      <c r="H1" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="14" t="s">
+      <c r="I1" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="9" t="s">
+      <c r="J1" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="9" t="s">
+      <c r="K1" s="12" t="s">
         <v>9</v>
       </c>
       <c r="L1" s="2"/>
@@ -4743,19 +4764,19 @@
       <c r="AA1" s="2"/>
     </row>
     <row r="2" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A2" s="10"/>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
+      <c r="A2" s="15"/>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
       <c r="F2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
-      <c r="I2" s="10"/>
-      <c r="J2" s="10"/>
-      <c r="K2" s="10"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
+      <c r="I2" s="15"/>
+      <c r="J2" s="15"/>
+      <c r="K2" s="15"/>
       <c r="L2" s="2"/>
       <c r="M2" s="2"/>
       <c r="N2" s="2"/>
@@ -4774,19 +4795,19 @@
       <c r="AA2" s="2"/>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A3" s="11"/>
-      <c r="B3" s="11"/>
-      <c r="C3" s="11"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="11"/>
+      <c r="A3" s="13"/>
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
       <c r="F3" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="G3" s="11"/>
-      <c r="H3" s="11"/>
-      <c r="I3" s="11"/>
-      <c r="J3" s="11"/>
-      <c r="K3" s="11"/>
+      <c r="G3" s="13"/>
+      <c r="H3" s="13"/>
+      <c r="I3" s="13"/>
+      <c r="J3" s="13"/>
+      <c r="K3" s="13"/>
       <c r="L3" s="2"/>
       <c r="M3" s="2"/>
       <c r="N3" s="2"/>
@@ -5369,32 +5390,32 @@
       <c r="AA15" s="2"/>
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A16" s="12" t="s">
+      <c r="A16" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="B16" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="C16" s="13" t="s">
+      <c r="C16" s="19" t="s">
         <v>70</v>
       </c>
-      <c r="D16" s="9">
+      <c r="D16" s="12">
         <v>2</v>
       </c>
-      <c r="E16" s="9">
+      <c r="E16" s="12">
         <v>223</v>
       </c>
-      <c r="F16" s="9" t="s">
+      <c r="F16" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="G16" s="9" t="s">
+      <c r="G16" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="H16" s="9" t="s">
+      <c r="H16" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="I16" s="9"/>
-      <c r="J16" s="9"/>
+      <c r="I16" s="12"/>
+      <c r="J16" s="12"/>
       <c r="K16" s="3" t="s">
         <v>72</v>
       </c>
@@ -5416,16 +5437,16 @@
       <c r="AA16" s="2"/>
     </row>
     <row r="17" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A17" s="11"/>
-      <c r="B17" s="11"/>
-      <c r="C17" s="11"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="11"/>
-      <c r="F17" s="11"/>
-      <c r="G17" s="11"/>
-      <c r="H17" s="11"/>
-      <c r="I17" s="11"/>
-      <c r="J17" s="11"/>
+      <c r="A17" s="13"/>
+      <c r="B17" s="13"/>
+      <c r="C17" s="13"/>
+      <c r="D17" s="13"/>
+      <c r="E17" s="13"/>
+      <c r="F17" s="13"/>
+      <c r="G17" s="13"/>
+      <c r="H17" s="13"/>
+      <c r="I17" s="13"/>
+      <c r="J17" s="13"/>
       <c r="K17" s="4" t="s">
         <v>73</v>
       </c>
@@ -5541,33 +5562,33 @@
       <c r="AA19" s="2"/>
     </row>
     <row r="20" spans="1:27" ht="108" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="12" t="s">
+      <c r="A20" s="14" t="s">
         <v>83</v>
       </c>
-      <c r="B20" s="9" t="s">
+      <c r="B20" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="C20" s="13" t="s">
+      <c r="C20" s="19" t="s">
         <v>85</v>
       </c>
-      <c r="D20" s="9">
+      <c r="D20" s="12">
         <v>12</v>
       </c>
-      <c r="E20" s="9">
+      <c r="E20" s="12">
         <v>1427</v>
       </c>
-      <c r="F20" s="9" t="s">
+      <c r="F20" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="G20" s="9" t="s">
+      <c r="G20" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="H20" s="9" t="s">
+      <c r="H20" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="I20" s="9"/>
-      <c r="J20" s="9"/>
-      <c r="K20" s="9" t="s">
+      <c r="I20" s="12"/>
+      <c r="J20" s="12"/>
+      <c r="K20" s="12" t="s">
         <v>82</v>
       </c>
       <c r="L20" s="2"/>
@@ -5588,17 +5609,17 @@
       <c r="AA20" s="2"/>
     </row>
     <row r="21" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="11"/>
-      <c r="B21" s="11"/>
-      <c r="C21" s="11"/>
-      <c r="D21" s="11"/>
-      <c r="E21" s="11"/>
-      <c r="F21" s="11"/>
-      <c r="G21" s="11"/>
-      <c r="H21" s="11"/>
-      <c r="I21" s="11"/>
-      <c r="J21" s="11"/>
-      <c r="K21" s="11"/>
+      <c r="A21" s="13"/>
+      <c r="B21" s="13"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="13"/>
+      <c r="E21" s="13"/>
+      <c r="F21" s="13"/>
+      <c r="G21" s="13"/>
+      <c r="H21" s="13"/>
+      <c r="I21" s="13"/>
+      <c r="J21" s="13"/>
+      <c r="K21" s="13"/>
       <c r="L21" s="2"/>
       <c r="M21" s="2"/>
       <c r="N21" s="2"/>
@@ -6218,32 +6239,32 @@
       <c r="AA34" s="2"/>
     </row>
     <row r="35" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="12" t="s">
+      <c r="A35" s="14" t="s">
         <v>145</v>
       </c>
-      <c r="B35" s="9" t="s">
+      <c r="B35" s="12" t="s">
         <v>146</v>
       </c>
-      <c r="C35" s="13" t="s">
+      <c r="C35" s="19" t="s">
         <v>147</v>
       </c>
-      <c r="D35" s="9">
+      <c r="D35" s="12">
         <v>44</v>
       </c>
-      <c r="E35" s="9">
+      <c r="E35" s="12">
         <v>3981</v>
       </c>
-      <c r="F35" s="9" t="s">
+      <c r="F35" s="12" t="s">
         <v>148</v>
       </c>
-      <c r="G35" s="9" t="s">
+      <c r="G35" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="H35" s="9" t="s">
+      <c r="H35" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="I35" s="9"/>
-      <c r="J35" s="9"/>
+      <c r="I35" s="12"/>
+      <c r="J35" s="12"/>
       <c r="K35" s="3" t="s">
         <v>149</v>
       </c>
@@ -6265,16 +6286,16 @@
       <c r="AA35" s="2"/>
     </row>
     <row r="36" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="10"/>
-      <c r="B36" s="10"/>
-      <c r="C36" s="10"/>
-      <c r="D36" s="10"/>
-      <c r="E36" s="10"/>
-      <c r="F36" s="10"/>
-      <c r="G36" s="10"/>
-      <c r="H36" s="10"/>
-      <c r="I36" s="10"/>
-      <c r="J36" s="10"/>
+      <c r="A36" s="15"/>
+      <c r="B36" s="15"/>
+      <c r="C36" s="15"/>
+      <c r="D36" s="15"/>
+      <c r="E36" s="15"/>
+      <c r="F36" s="15"/>
+      <c r="G36" s="15"/>
+      <c r="H36" s="15"/>
+      <c r="I36" s="15"/>
+      <c r="J36" s="15"/>
       <c r="K36" s="3" t="s">
         <v>150</v>
       </c>
@@ -6296,16 +6317,16 @@
       <c r="AA36" s="2"/>
     </row>
     <row r="37" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="10"/>
-      <c r="B37" s="10"/>
-      <c r="C37" s="10"/>
-      <c r="D37" s="10"/>
-      <c r="E37" s="10"/>
-      <c r="F37" s="10"/>
-      <c r="G37" s="10"/>
-      <c r="H37" s="10"/>
-      <c r="I37" s="10"/>
-      <c r="J37" s="10"/>
+      <c r="A37" s="15"/>
+      <c r="B37" s="15"/>
+      <c r="C37" s="15"/>
+      <c r="D37" s="15"/>
+      <c r="E37" s="15"/>
+      <c r="F37" s="15"/>
+      <c r="G37" s="15"/>
+      <c r="H37" s="15"/>
+      <c r="I37" s="15"/>
+      <c r="J37" s="15"/>
       <c r="K37" s="3"/>
       <c r="L37" s="2"/>
       <c r="M37" s="2"/>
@@ -6325,16 +6346,16 @@
       <c r="AA37" s="2"/>
     </row>
     <row r="38" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="11"/>
-      <c r="B38" s="11"/>
-      <c r="C38" s="11"/>
-      <c r="D38" s="11"/>
-      <c r="E38" s="11"/>
-      <c r="F38" s="11"/>
-      <c r="G38" s="11"/>
-      <c r="H38" s="11"/>
-      <c r="I38" s="11"/>
-      <c r="J38" s="11"/>
+      <c r="A38" s="13"/>
+      <c r="B38" s="13"/>
+      <c r="C38" s="13"/>
+      <c r="D38" s="13"/>
+      <c r="E38" s="13"/>
+      <c r="F38" s="13"/>
+      <c r="G38" s="13"/>
+      <c r="H38" s="13"/>
+      <c r="I38" s="13"/>
+      <c r="J38" s="13"/>
       <c r="K38" s="4" t="s">
         <v>151</v>
       </c>
@@ -6632,28 +6653,28 @@
       <c r="AA44" s="2"/>
     </row>
     <row r="45" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="12" t="s">
+      <c r="A45" s="14" t="s">
         <v>179</v>
       </c>
-      <c r="B45" s="9" t="s">
+      <c r="B45" s="12" t="s">
         <v>180</v>
       </c>
-      <c r="C45" s="13" t="s">
+      <c r="C45" s="19" t="s">
         <v>181</v>
       </c>
-      <c r="D45" s="9">
+      <c r="D45" s="12">
         <v>48</v>
       </c>
-      <c r="E45" s="9">
+      <c r="E45" s="12">
         <v>10207</v>
       </c>
-      <c r="F45" s="9" t="s">
+      <c r="F45" s="12" t="s">
         <v>182</v>
       </c>
-      <c r="G45" s="9"/>
-      <c r="H45" s="9"/>
-      <c r="I45" s="9"/>
-      <c r="J45" s="9"/>
+      <c r="G45" s="12"/>
+      <c r="H45" s="12"/>
+      <c r="I45" s="12"/>
+      <c r="J45" s="12"/>
       <c r="K45" s="3" t="s">
         <v>183</v>
       </c>
@@ -6675,16 +6696,16 @@
       <c r="AA45" s="2"/>
     </row>
     <row r="46" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="10"/>
-      <c r="B46" s="10"/>
-      <c r="C46" s="10"/>
-      <c r="D46" s="10"/>
-      <c r="E46" s="10"/>
-      <c r="F46" s="10"/>
-      <c r="G46" s="10"/>
-      <c r="H46" s="10"/>
-      <c r="I46" s="10"/>
-      <c r="J46" s="10"/>
+      <c r="A46" s="15"/>
+      <c r="B46" s="15"/>
+      <c r="C46" s="15"/>
+      <c r="D46" s="15"/>
+      <c r="E46" s="15"/>
+      <c r="F46" s="15"/>
+      <c r="G46" s="15"/>
+      <c r="H46" s="15"/>
+      <c r="I46" s="15"/>
+      <c r="J46" s="15"/>
       <c r="K46" s="3" t="s">
         <v>184</v>
       </c>
@@ -6706,16 +6727,16 @@
       <c r="AA46" s="2"/>
     </row>
     <row r="47" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="10"/>
-      <c r="B47" s="10"/>
-      <c r="C47" s="10"/>
-      <c r="D47" s="10"/>
-      <c r="E47" s="10"/>
-      <c r="F47" s="10"/>
-      <c r="G47" s="10"/>
-      <c r="H47" s="10"/>
-      <c r="I47" s="10"/>
-      <c r="J47" s="10"/>
+      <c r="A47" s="15"/>
+      <c r="B47" s="15"/>
+      <c r="C47" s="15"/>
+      <c r="D47" s="15"/>
+      <c r="E47" s="15"/>
+      <c r="F47" s="15"/>
+      <c r="G47" s="15"/>
+      <c r="H47" s="15"/>
+      <c r="I47" s="15"/>
+      <c r="J47" s="15"/>
       <c r="K47" s="3" t="s">
         <v>185</v>
       </c>
@@ -6737,16 +6758,16 @@
       <c r="AA47" s="2"/>
     </row>
     <row r="48" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="10"/>
-      <c r="B48" s="10"/>
-      <c r="C48" s="10"/>
-      <c r="D48" s="10"/>
-      <c r="E48" s="10"/>
-      <c r="F48" s="10"/>
-      <c r="G48" s="10"/>
-      <c r="H48" s="10"/>
-      <c r="I48" s="10"/>
-      <c r="J48" s="10"/>
+      <c r="A48" s="15"/>
+      <c r="B48" s="15"/>
+      <c r="C48" s="15"/>
+      <c r="D48" s="15"/>
+      <c r="E48" s="15"/>
+      <c r="F48" s="15"/>
+      <c r="G48" s="15"/>
+      <c r="H48" s="15"/>
+      <c r="I48" s="15"/>
+      <c r="J48" s="15"/>
       <c r="K48" s="3" t="s">
         <v>186</v>
       </c>
@@ -6768,16 +6789,16 @@
       <c r="AA48" s="2"/>
     </row>
     <row r="49" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="10"/>
-      <c r="B49" s="10"/>
-      <c r="C49" s="10"/>
-      <c r="D49" s="10"/>
-      <c r="E49" s="10"/>
-      <c r="F49" s="10"/>
-      <c r="G49" s="10"/>
-      <c r="H49" s="10"/>
-      <c r="I49" s="10"/>
-      <c r="J49" s="10"/>
+      <c r="A49" s="15"/>
+      <c r="B49" s="15"/>
+      <c r="C49" s="15"/>
+      <c r="D49" s="15"/>
+      <c r="E49" s="15"/>
+      <c r="F49" s="15"/>
+      <c r="G49" s="15"/>
+      <c r="H49" s="15"/>
+      <c r="I49" s="15"/>
+      <c r="J49" s="15"/>
       <c r="K49" s="3" t="s">
         <v>187</v>
       </c>
@@ -6799,16 +6820,16 @@
       <c r="AA49" s="2"/>
     </row>
     <row r="50" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="10"/>
-      <c r="B50" s="10"/>
-      <c r="C50" s="10"/>
-      <c r="D50" s="10"/>
-      <c r="E50" s="10"/>
-      <c r="F50" s="10"/>
-      <c r="G50" s="10"/>
-      <c r="H50" s="10"/>
-      <c r="I50" s="10"/>
-      <c r="J50" s="10"/>
+      <c r="A50" s="15"/>
+      <c r="B50" s="15"/>
+      <c r="C50" s="15"/>
+      <c r="D50" s="15"/>
+      <c r="E50" s="15"/>
+      <c r="F50" s="15"/>
+      <c r="G50" s="15"/>
+      <c r="H50" s="15"/>
+      <c r="I50" s="15"/>
+      <c r="J50" s="15"/>
       <c r="K50" s="3" t="s">
         <v>188</v>
       </c>
@@ -6830,16 +6851,16 @@
       <c r="AA50" s="2"/>
     </row>
     <row r="51" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="10"/>
-      <c r="B51" s="10"/>
-      <c r="C51" s="10"/>
-      <c r="D51" s="10"/>
-      <c r="E51" s="10"/>
-      <c r="F51" s="10"/>
-      <c r="G51" s="10"/>
-      <c r="H51" s="10"/>
-      <c r="I51" s="10"/>
-      <c r="J51" s="10"/>
+      <c r="A51" s="15"/>
+      <c r="B51" s="15"/>
+      <c r="C51" s="15"/>
+      <c r="D51" s="15"/>
+      <c r="E51" s="15"/>
+      <c r="F51" s="15"/>
+      <c r="G51" s="15"/>
+      <c r="H51" s="15"/>
+      <c r="I51" s="15"/>
+      <c r="J51" s="15"/>
       <c r="K51" s="3" t="s">
         <v>189</v>
       </c>
@@ -6861,16 +6882,16 @@
       <c r="AA51" s="2"/>
     </row>
     <row r="52" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="10"/>
-      <c r="B52" s="10"/>
-      <c r="C52" s="10"/>
-      <c r="D52" s="10"/>
-      <c r="E52" s="10"/>
-      <c r="F52" s="10"/>
-      <c r="G52" s="10"/>
-      <c r="H52" s="10"/>
-      <c r="I52" s="10"/>
-      <c r="J52" s="10"/>
+      <c r="A52" s="15"/>
+      <c r="B52" s="15"/>
+      <c r="C52" s="15"/>
+      <c r="D52" s="15"/>
+      <c r="E52" s="15"/>
+      <c r="F52" s="15"/>
+      <c r="G52" s="15"/>
+      <c r="H52" s="15"/>
+      <c r="I52" s="15"/>
+      <c r="J52" s="15"/>
       <c r="K52" s="3" t="s">
         <v>190</v>
       </c>
@@ -6892,16 +6913,16 @@
       <c r="AA52" s="2"/>
     </row>
     <row r="53" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="10"/>
-      <c r="B53" s="10"/>
-      <c r="C53" s="10"/>
-      <c r="D53" s="10"/>
-      <c r="E53" s="10"/>
-      <c r="F53" s="10"/>
-      <c r="G53" s="10"/>
-      <c r="H53" s="10"/>
-      <c r="I53" s="10"/>
-      <c r="J53" s="10"/>
+      <c r="A53" s="15"/>
+      <c r="B53" s="15"/>
+      <c r="C53" s="15"/>
+      <c r="D53" s="15"/>
+      <c r="E53" s="15"/>
+      <c r="F53" s="15"/>
+      <c r="G53" s="15"/>
+      <c r="H53" s="15"/>
+      <c r="I53" s="15"/>
+      <c r="J53" s="15"/>
       <c r="K53" s="3" t="s">
         <v>191</v>
       </c>
@@ -6923,16 +6944,16 @@
       <c r="AA53" s="2"/>
     </row>
     <row r="54" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="10"/>
-      <c r="B54" s="10"/>
-      <c r="C54" s="10"/>
-      <c r="D54" s="10"/>
-      <c r="E54" s="10"/>
-      <c r="F54" s="10"/>
-      <c r="G54" s="10"/>
-      <c r="H54" s="10"/>
-      <c r="I54" s="10"/>
-      <c r="J54" s="10"/>
+      <c r="A54" s="15"/>
+      <c r="B54" s="15"/>
+      <c r="C54" s="15"/>
+      <c r="D54" s="15"/>
+      <c r="E54" s="15"/>
+      <c r="F54" s="15"/>
+      <c r="G54" s="15"/>
+      <c r="H54" s="15"/>
+      <c r="I54" s="15"/>
+      <c r="J54" s="15"/>
       <c r="K54" s="3" t="s">
         <v>192</v>
       </c>
@@ -6954,16 +6975,16 @@
       <c r="AA54" s="2"/>
     </row>
     <row r="55" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="10"/>
-      <c r="B55" s="10"/>
-      <c r="C55" s="10"/>
-      <c r="D55" s="10"/>
-      <c r="E55" s="10"/>
-      <c r="F55" s="10"/>
-      <c r="G55" s="10"/>
-      <c r="H55" s="10"/>
-      <c r="I55" s="10"/>
-      <c r="J55" s="10"/>
+      <c r="A55" s="15"/>
+      <c r="B55" s="15"/>
+      <c r="C55" s="15"/>
+      <c r="D55" s="15"/>
+      <c r="E55" s="15"/>
+      <c r="F55" s="15"/>
+      <c r="G55" s="15"/>
+      <c r="H55" s="15"/>
+      <c r="I55" s="15"/>
+      <c r="J55" s="15"/>
       <c r="K55" s="3" t="s">
         <v>193</v>
       </c>
@@ -6985,16 +7006,16 @@
       <c r="AA55" s="2"/>
     </row>
     <row r="56" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="10"/>
-      <c r="B56" s="10"/>
-      <c r="C56" s="10"/>
-      <c r="D56" s="10"/>
-      <c r="E56" s="10"/>
-      <c r="F56" s="10"/>
-      <c r="G56" s="10"/>
-      <c r="H56" s="10"/>
-      <c r="I56" s="10"/>
-      <c r="J56" s="10"/>
+      <c r="A56" s="15"/>
+      <c r="B56" s="15"/>
+      <c r="C56" s="15"/>
+      <c r="D56" s="15"/>
+      <c r="E56" s="15"/>
+      <c r="F56" s="15"/>
+      <c r="G56" s="15"/>
+      <c r="H56" s="15"/>
+      <c r="I56" s="15"/>
+      <c r="J56" s="15"/>
       <c r="K56" s="3" t="s">
         <v>194</v>
       </c>
@@ -7016,16 +7037,16 @@
       <c r="AA56" s="2"/>
     </row>
     <row r="57" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="10"/>
-      <c r="B57" s="10"/>
-      <c r="C57" s="10"/>
-      <c r="D57" s="10"/>
-      <c r="E57" s="10"/>
-      <c r="F57" s="10"/>
-      <c r="G57" s="10"/>
-      <c r="H57" s="10"/>
-      <c r="I57" s="10"/>
-      <c r="J57" s="10"/>
+      <c r="A57" s="15"/>
+      <c r="B57" s="15"/>
+      <c r="C57" s="15"/>
+      <c r="D57" s="15"/>
+      <c r="E57" s="15"/>
+      <c r="F57" s="15"/>
+      <c r="G57" s="15"/>
+      <c r="H57" s="15"/>
+      <c r="I57" s="15"/>
+      <c r="J57" s="15"/>
       <c r="K57" s="3" t="s">
         <v>195</v>
       </c>
@@ -7047,16 +7068,16 @@
       <c r="AA57" s="2"/>
     </row>
     <row r="58" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="10"/>
-      <c r="B58" s="10"/>
-      <c r="C58" s="10"/>
-      <c r="D58" s="10"/>
-      <c r="E58" s="10"/>
-      <c r="F58" s="10"/>
-      <c r="G58" s="10"/>
-      <c r="H58" s="10"/>
-      <c r="I58" s="10"/>
-      <c r="J58" s="10"/>
+      <c r="A58" s="15"/>
+      <c r="B58" s="15"/>
+      <c r="C58" s="15"/>
+      <c r="D58" s="15"/>
+      <c r="E58" s="15"/>
+      <c r="F58" s="15"/>
+      <c r="G58" s="15"/>
+      <c r="H58" s="15"/>
+      <c r="I58" s="15"/>
+      <c r="J58" s="15"/>
       <c r="K58" s="3" t="s">
         <v>196</v>
       </c>
@@ -7078,16 +7099,16 @@
       <c r="AA58" s="2"/>
     </row>
     <row r="59" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="10"/>
-      <c r="B59" s="10"/>
-      <c r="C59" s="10"/>
-      <c r="D59" s="10"/>
-      <c r="E59" s="10"/>
-      <c r="F59" s="10"/>
-      <c r="G59" s="10"/>
-      <c r="H59" s="10"/>
-      <c r="I59" s="10"/>
-      <c r="J59" s="10"/>
+      <c r="A59" s="15"/>
+      <c r="B59" s="15"/>
+      <c r="C59" s="15"/>
+      <c r="D59" s="15"/>
+      <c r="E59" s="15"/>
+      <c r="F59" s="15"/>
+      <c r="G59" s="15"/>
+      <c r="H59" s="15"/>
+      <c r="I59" s="15"/>
+      <c r="J59" s="15"/>
       <c r="K59" s="3" t="s">
         <v>197</v>
       </c>
@@ -7109,16 +7130,16 @@
       <c r="AA59" s="2"/>
     </row>
     <row r="60" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="10"/>
-      <c r="B60" s="10"/>
-      <c r="C60" s="10"/>
-      <c r="D60" s="10"/>
-      <c r="E60" s="10"/>
-      <c r="F60" s="10"/>
-      <c r="G60" s="10"/>
-      <c r="H60" s="10"/>
-      <c r="I60" s="10"/>
-      <c r="J60" s="10"/>
+      <c r="A60" s="15"/>
+      <c r="B60" s="15"/>
+      <c r="C60" s="15"/>
+      <c r="D60" s="15"/>
+      <c r="E60" s="15"/>
+      <c r="F60" s="15"/>
+      <c r="G60" s="15"/>
+      <c r="H60" s="15"/>
+      <c r="I60" s="15"/>
+      <c r="J60" s="15"/>
       <c r="K60" s="3" t="s">
         <v>198</v>
       </c>
@@ -7140,16 +7161,16 @@
       <c r="AA60" s="2"/>
     </row>
     <row r="61" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="10"/>
-      <c r="B61" s="10"/>
-      <c r="C61" s="10"/>
-      <c r="D61" s="10"/>
-      <c r="E61" s="10"/>
-      <c r="F61" s="10"/>
-      <c r="G61" s="10"/>
-      <c r="H61" s="10"/>
-      <c r="I61" s="10"/>
-      <c r="J61" s="10"/>
+      <c r="A61" s="15"/>
+      <c r="B61" s="15"/>
+      <c r="C61" s="15"/>
+      <c r="D61" s="15"/>
+      <c r="E61" s="15"/>
+      <c r="F61" s="15"/>
+      <c r="G61" s="15"/>
+      <c r="H61" s="15"/>
+      <c r="I61" s="15"/>
+      <c r="J61" s="15"/>
       <c r="K61" s="3" t="s">
         <v>199</v>
       </c>
@@ -7171,16 +7192,16 @@
       <c r="AA61" s="2"/>
     </row>
     <row r="62" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="10"/>
-      <c r="B62" s="10"/>
-      <c r="C62" s="10"/>
-      <c r="D62" s="10"/>
-      <c r="E62" s="10"/>
-      <c r="F62" s="10"/>
-      <c r="G62" s="10"/>
-      <c r="H62" s="10"/>
-      <c r="I62" s="10"/>
-      <c r="J62" s="10"/>
+      <c r="A62" s="15"/>
+      <c r="B62" s="15"/>
+      <c r="C62" s="15"/>
+      <c r="D62" s="15"/>
+      <c r="E62" s="15"/>
+      <c r="F62" s="15"/>
+      <c r="G62" s="15"/>
+      <c r="H62" s="15"/>
+      <c r="I62" s="15"/>
+      <c r="J62" s="15"/>
       <c r="K62" s="3" t="s">
         <v>200</v>
       </c>
@@ -7202,16 +7223,16 @@
       <c r="AA62" s="2"/>
     </row>
     <row r="63" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="10"/>
-      <c r="B63" s="10"/>
-      <c r="C63" s="10"/>
-      <c r="D63" s="10"/>
-      <c r="E63" s="10"/>
-      <c r="F63" s="10"/>
-      <c r="G63" s="10"/>
-      <c r="H63" s="10"/>
-      <c r="I63" s="10"/>
-      <c r="J63" s="10"/>
+      <c r="A63" s="15"/>
+      <c r="B63" s="15"/>
+      <c r="C63" s="15"/>
+      <c r="D63" s="15"/>
+      <c r="E63" s="15"/>
+      <c r="F63" s="15"/>
+      <c r="G63" s="15"/>
+      <c r="H63" s="15"/>
+      <c r="I63" s="15"/>
+      <c r="J63" s="15"/>
       <c r="K63" s="3" t="s">
         <v>201</v>
       </c>
@@ -7233,16 +7254,16 @@
       <c r="AA63" s="2"/>
     </row>
     <row r="64" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="10"/>
-      <c r="B64" s="10"/>
-      <c r="C64" s="10"/>
-      <c r="D64" s="10"/>
-      <c r="E64" s="10"/>
-      <c r="F64" s="10"/>
-      <c r="G64" s="10"/>
-      <c r="H64" s="10"/>
-      <c r="I64" s="10"/>
-      <c r="J64" s="10"/>
+      <c r="A64" s="15"/>
+      <c r="B64" s="15"/>
+      <c r="C64" s="15"/>
+      <c r="D64" s="15"/>
+      <c r="E64" s="15"/>
+      <c r="F64" s="15"/>
+      <c r="G64" s="15"/>
+      <c r="H64" s="15"/>
+      <c r="I64" s="15"/>
+      <c r="J64" s="15"/>
       <c r="K64" s="3" t="s">
         <v>202</v>
       </c>
@@ -7264,16 +7285,16 @@
       <c r="AA64" s="2"/>
     </row>
     <row r="65" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="10"/>
-      <c r="B65" s="10"/>
-      <c r="C65" s="10"/>
-      <c r="D65" s="10"/>
-      <c r="E65" s="10"/>
-      <c r="F65" s="10"/>
-      <c r="G65" s="10"/>
-      <c r="H65" s="10"/>
-      <c r="I65" s="10"/>
-      <c r="J65" s="10"/>
+      <c r="A65" s="15"/>
+      <c r="B65" s="15"/>
+      <c r="C65" s="15"/>
+      <c r="D65" s="15"/>
+      <c r="E65" s="15"/>
+      <c r="F65" s="15"/>
+      <c r="G65" s="15"/>
+      <c r="H65" s="15"/>
+      <c r="I65" s="15"/>
+      <c r="J65" s="15"/>
       <c r="K65" s="3" t="s">
         <v>203</v>
       </c>
@@ -7295,16 +7316,16 @@
       <c r="AA65" s="2"/>
     </row>
     <row r="66" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="10"/>
-      <c r="B66" s="10"/>
-      <c r="C66" s="10"/>
-      <c r="D66" s="10"/>
-      <c r="E66" s="10"/>
-      <c r="F66" s="10"/>
-      <c r="G66" s="10"/>
-      <c r="H66" s="10"/>
-      <c r="I66" s="10"/>
-      <c r="J66" s="10"/>
+      <c r="A66" s="15"/>
+      <c r="B66" s="15"/>
+      <c r="C66" s="15"/>
+      <c r="D66" s="15"/>
+      <c r="E66" s="15"/>
+      <c r="F66" s="15"/>
+      <c r="G66" s="15"/>
+      <c r="H66" s="15"/>
+      <c r="I66" s="15"/>
+      <c r="J66" s="15"/>
       <c r="K66" s="3" t="s">
         <v>204</v>
       </c>
@@ -7326,16 +7347,16 @@
       <c r="AA66" s="2"/>
     </row>
     <row r="67" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="10"/>
-      <c r="B67" s="10"/>
-      <c r="C67" s="10"/>
-      <c r="D67" s="10"/>
-      <c r="E67" s="10"/>
-      <c r="F67" s="10"/>
-      <c r="G67" s="10"/>
-      <c r="H67" s="10"/>
-      <c r="I67" s="10"/>
-      <c r="J67" s="10"/>
+      <c r="A67" s="15"/>
+      <c r="B67" s="15"/>
+      <c r="C67" s="15"/>
+      <c r="D67" s="15"/>
+      <c r="E67" s="15"/>
+      <c r="F67" s="15"/>
+      <c r="G67" s="15"/>
+      <c r="H67" s="15"/>
+      <c r="I67" s="15"/>
+      <c r="J67" s="15"/>
       <c r="K67" s="3" t="s">
         <v>205</v>
       </c>
@@ -7357,16 +7378,16 @@
       <c r="AA67" s="2"/>
     </row>
     <row r="68" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="10"/>
-      <c r="B68" s="10"/>
-      <c r="C68" s="10"/>
-      <c r="D68" s="10"/>
-      <c r="E68" s="10"/>
-      <c r="F68" s="10"/>
-      <c r="G68" s="10"/>
-      <c r="H68" s="10"/>
-      <c r="I68" s="10"/>
-      <c r="J68" s="10"/>
+      <c r="A68" s="15"/>
+      <c r="B68" s="15"/>
+      <c r="C68" s="15"/>
+      <c r="D68" s="15"/>
+      <c r="E68" s="15"/>
+      <c r="F68" s="15"/>
+      <c r="G68" s="15"/>
+      <c r="H68" s="15"/>
+      <c r="I68" s="15"/>
+      <c r="J68" s="15"/>
       <c r="K68" s="3" t="s">
         <v>206</v>
       </c>
@@ -7388,16 +7409,16 @@
       <c r="AA68" s="2"/>
     </row>
     <row r="69" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="10"/>
-      <c r="B69" s="10"/>
-      <c r="C69" s="10"/>
-      <c r="D69" s="10"/>
-      <c r="E69" s="10"/>
-      <c r="F69" s="10"/>
-      <c r="G69" s="10"/>
-      <c r="H69" s="10"/>
-      <c r="I69" s="10"/>
-      <c r="J69" s="10"/>
+      <c r="A69" s="15"/>
+      <c r="B69" s="15"/>
+      <c r="C69" s="15"/>
+      <c r="D69" s="15"/>
+      <c r="E69" s="15"/>
+      <c r="F69" s="15"/>
+      <c r="G69" s="15"/>
+      <c r="H69" s="15"/>
+      <c r="I69" s="15"/>
+      <c r="J69" s="15"/>
       <c r="K69" s="3" t="s">
         <v>207</v>
       </c>
@@ -7419,16 +7440,16 @@
       <c r="AA69" s="2"/>
     </row>
     <row r="70" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="10"/>
-      <c r="B70" s="10"/>
-      <c r="C70" s="10"/>
-      <c r="D70" s="10"/>
-      <c r="E70" s="10"/>
-      <c r="F70" s="10"/>
-      <c r="G70" s="10"/>
-      <c r="H70" s="10"/>
-      <c r="I70" s="10"/>
-      <c r="J70" s="10"/>
+      <c r="A70" s="15"/>
+      <c r="B70" s="15"/>
+      <c r="C70" s="15"/>
+      <c r="D70" s="15"/>
+      <c r="E70" s="15"/>
+      <c r="F70" s="15"/>
+      <c r="G70" s="15"/>
+      <c r="H70" s="15"/>
+      <c r="I70" s="15"/>
+      <c r="J70" s="15"/>
       <c r="K70" s="3"/>
       <c r="L70" s="2"/>
       <c r="M70" s="2"/>
@@ -7447,17 +7468,17 @@
       <c r="Z70" s="2"/>
       <c r="AA70" s="2"/>
     </row>
-    <row r="71" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="11"/>
-      <c r="B71" s="11"/>
-      <c r="C71" s="11"/>
-      <c r="D71" s="11"/>
-      <c r="E71" s="11"/>
-      <c r="F71" s="11"/>
-      <c r="G71" s="11"/>
-      <c r="H71" s="11"/>
-      <c r="I71" s="11"/>
-      <c r="J71" s="11"/>
+    <row r="71" spans="1:27" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A71" s="13"/>
+      <c r="B71" s="13"/>
+      <c r="C71" s="13"/>
+      <c r="D71" s="13"/>
+      <c r="E71" s="13"/>
+      <c r="F71" s="13"/>
+      <c r="G71" s="13"/>
+      <c r="H71" s="13"/>
+      <c r="I71" s="13"/>
+      <c r="J71" s="13"/>
       <c r="K71" s="4" t="s">
         <v>208</v>
       </c>
@@ -7478,35 +7499,33 @@
       <c r="Z71" s="2"/>
       <c r="AA71" s="2"/>
     </row>
-    <row r="72" spans="1:27" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="5" t="s">
-        <v>209</v>
-      </c>
-      <c r="B72" s="4" t="s">
-        <v>210</v>
-      </c>
-      <c r="C72" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="D72" s="4">
-        <v>1</v>
-      </c>
-      <c r="E72" s="4">
-        <v>332</v>
-      </c>
-      <c r="F72" s="4" t="s">
-        <v>212</v>
-      </c>
-      <c r="G72" s="4" t="s">
+    <row r="72" spans="1:27" s="24" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A72" s="22"/>
+      <c r="B72" s="23" t="s">
+        <v>520</v>
+      </c>
+      <c r="C72" s="23" t="s">
+        <v>519</v>
+      </c>
+      <c r="D72" s="23">
+        <v>14</v>
+      </c>
+      <c r="E72" s="23">
+        <v>2629</v>
+      </c>
+      <c r="F72" s="23" t="s">
+        <v>518</v>
+      </c>
+      <c r="G72" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="H72" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="I72" s="4"/>
-      <c r="J72" s="4"/>
+      <c r="H72" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="I72" s="23"/>
+      <c r="J72" s="23"/>
       <c r="K72" s="4" t="s">
-        <v>213</v>
+        <v>521</v>
       </c>
       <c r="L72" s="2"/>
       <c r="M72" s="2"/>
@@ -7526,32 +7545,34 @@
       <c r="AA72" s="2"/>
     </row>
     <row r="73" spans="1:27" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A73" s="5"/>
-      <c r="B73" s="19" t="s">
-        <v>514</v>
-      </c>
-      <c r="C73" s="21" t="s">
-        <v>515</v>
+      <c r="A73" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="B73" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="C73" s="6" t="s">
+        <v>211</v>
       </c>
       <c r="D73" s="4">
         <v>1</v>
       </c>
       <c r="E73" s="4">
-        <v>300</v>
-      </c>
-      <c r="F73" s="20" t="s">
-        <v>516</v>
-      </c>
-      <c r="G73" s="20" t="s">
+        <v>332</v>
+      </c>
+      <c r="F73" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="G73" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="H73" s="20" t="s">
-        <v>17</v>
+      <c r="H73" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="I73" s="4"/>
       <c r="J73" s="4"/>
-      <c r="K73" s="20" t="s">
-        <v>517</v>
+      <c r="K73" s="4" t="s">
+        <v>213</v>
       </c>
       <c r="L73" s="2"/>
       <c r="M73" s="2"/>
@@ -7571,30 +7592,32 @@
       <c r="AA73" s="2"/>
     </row>
     <row r="74" spans="1:27" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A74" s="5" t="s">
-        <v>214</v>
-      </c>
-      <c r="B74" s="4" t="s">
-        <v>215</v>
-      </c>
-      <c r="C74" s="6" t="s">
-        <v>216</v>
+      <c r="A74" s="5"/>
+      <c r="B74" s="9" t="s">
+        <v>514</v>
+      </c>
+      <c r="C74" s="11" t="s">
+        <v>515</v>
       </c>
       <c r="D74" s="4">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="E74" s="4">
-        <v>1129</v>
-      </c>
-      <c r="F74" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="G74" s="4"/>
-      <c r="H74" s="4"/>
+        <v>300</v>
+      </c>
+      <c r="F74" s="10" t="s">
+        <v>516</v>
+      </c>
+      <c r="G74" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="H74" s="10" t="s">
+        <v>17</v>
+      </c>
       <c r="I74" s="4"/>
       <c r="J74" s="4"/>
-      <c r="K74" s="4" t="s">
-        <v>218</v>
+      <c r="K74" s="10" t="s">
+        <v>517</v>
       </c>
       <c r="L74" s="2"/>
       <c r="M74" s="2"/>
@@ -7613,35 +7636,31 @@
       <c r="Z74" s="2"/>
       <c r="AA74" s="2"/>
     </row>
-    <row r="75" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="12" t="s">
-        <v>219</v>
-      </c>
-      <c r="B75" s="9" t="s">
-        <v>220</v>
-      </c>
-      <c r="C75" s="13" t="s">
-        <v>221</v>
-      </c>
-      <c r="D75" s="9">
-        <v>10</v>
-      </c>
-      <c r="E75" s="9">
-        <v>1153</v>
-      </c>
-      <c r="F75" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="G75" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="H75" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="I75" s="9"/>
-      <c r="J75" s="9"/>
-      <c r="K75" s="3" t="s">
-        <v>223</v>
+    <row r="75" spans="1:27" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A75" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="B75" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="C75" s="6" t="s">
+        <v>216</v>
+      </c>
+      <c r="D75" s="4">
+        <v>11</v>
+      </c>
+      <c r="E75" s="4">
+        <v>1129</v>
+      </c>
+      <c r="F75" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="G75" s="4"/>
+      <c r="H75" s="4"/>
+      <c r="I75" s="4"/>
+      <c r="J75" s="4"/>
+      <c r="K75" s="4" t="s">
+        <v>218</v>
       </c>
       <c r="L75" s="2"/>
       <c r="M75" s="2"/>
@@ -7661,18 +7680,34 @@
       <c r="AA75" s="2"/>
     </row>
     <row r="76" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="10"/>
-      <c r="B76" s="10"/>
-      <c r="C76" s="10"/>
-      <c r="D76" s="10"/>
-      <c r="E76" s="10"/>
-      <c r="F76" s="10"/>
-      <c r="G76" s="10"/>
-      <c r="H76" s="10"/>
-      <c r="I76" s="10"/>
-      <c r="J76" s="10"/>
+      <c r="A76" s="14" t="s">
+        <v>219</v>
+      </c>
+      <c r="B76" s="12" t="s">
+        <v>220</v>
+      </c>
+      <c r="C76" s="19" t="s">
+        <v>221</v>
+      </c>
+      <c r="D76" s="12">
+        <v>10</v>
+      </c>
+      <c r="E76" s="12">
+        <v>1153</v>
+      </c>
+      <c r="F76" s="12" t="s">
+        <v>222</v>
+      </c>
+      <c r="G76" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H76" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="I76" s="12"/>
+      <c r="J76" s="12"/>
       <c r="K76" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="L76" s="2"/>
       <c r="M76" s="2"/>
@@ -7692,18 +7727,18 @@
       <c r="AA76" s="2"/>
     </row>
     <row r="77" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="10"/>
-      <c r="B77" s="10"/>
-      <c r="C77" s="10"/>
-      <c r="D77" s="10"/>
-      <c r="E77" s="10"/>
-      <c r="F77" s="10"/>
-      <c r="G77" s="10"/>
-      <c r="H77" s="10"/>
-      <c r="I77" s="10"/>
-      <c r="J77" s="10"/>
+      <c r="A77" s="15"/>
+      <c r="B77" s="15"/>
+      <c r="C77" s="15"/>
+      <c r="D77" s="15"/>
+      <c r="E77" s="15"/>
+      <c r="F77" s="15"/>
+      <c r="G77" s="15"/>
+      <c r="H77" s="15"/>
+      <c r="I77" s="15"/>
+      <c r="J77" s="15"/>
       <c r="K77" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L77" s="2"/>
       <c r="M77" s="2"/>
@@ -7723,16 +7758,19 @@
       <c r="AA77" s="2"/>
     </row>
     <row r="78" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="10"/>
-      <c r="B78" s="10"/>
-      <c r="C78" s="10"/>
-      <c r="D78" s="10"/>
-      <c r="E78" s="10"/>
-      <c r="F78" s="10"/>
-      <c r="G78" s="10"/>
-      <c r="H78" s="10"/>
-      <c r="I78" s="10"/>
-      <c r="J78" s="10"/>
+      <c r="A78" s="15"/>
+      <c r="B78" s="15"/>
+      <c r="C78" s="15"/>
+      <c r="D78" s="15"/>
+      <c r="E78" s="15"/>
+      <c r="F78" s="15"/>
+      <c r="G78" s="15"/>
+      <c r="H78" s="15"/>
+      <c r="I78" s="15"/>
+      <c r="J78" s="15"/>
+      <c r="K78" s="3" t="s">
+        <v>225</v>
+      </c>
       <c r="L78" s="2"/>
       <c r="M78" s="2"/>
       <c r="N78" s="2"/>
@@ -7751,19 +7789,16 @@
       <c r="AA78" s="2"/>
     </row>
     <row r="79" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="11"/>
-      <c r="B79" s="11"/>
-      <c r="C79" s="11"/>
-      <c r="D79" s="11"/>
-      <c r="E79" s="11"/>
-      <c r="F79" s="11"/>
-      <c r="G79" s="11"/>
-      <c r="H79" s="11"/>
-      <c r="I79" s="11"/>
-      <c r="J79" s="11"/>
-      <c r="K79" s="4" t="s">
-        <v>226</v>
-      </c>
+      <c r="A79" s="15"/>
+      <c r="B79" s="15"/>
+      <c r="C79" s="15"/>
+      <c r="D79" s="15"/>
+      <c r="E79" s="15"/>
+      <c r="F79" s="15"/>
+      <c r="G79" s="15"/>
+      <c r="H79" s="15"/>
+      <c r="I79" s="15"/>
+      <c r="J79" s="15"/>
       <c r="L79" s="2"/>
       <c r="M79" s="2"/>
       <c r="N79" s="2"/>
@@ -7782,32 +7817,18 @@
       <c r="AA79" s="2"/>
     </row>
     <row r="80" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="12" t="s">
-        <v>227</v>
-      </c>
-      <c r="B80" s="9" t="s">
-        <v>228</v>
-      </c>
-      <c r="C80" s="13" t="s">
-        <v>229</v>
-      </c>
-      <c r="D80" s="9">
-        <v>44</v>
-      </c>
-      <c r="E80" s="9">
-        <v>3709</v>
-      </c>
-      <c r="F80" s="9" t="s">
-        <v>230</v>
-      </c>
-      <c r="G80" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="H80" s="9"/>
-      <c r="I80" s="9"/>
-      <c r="J80" s="9"/>
-      <c r="K80" s="3" t="s">
-        <v>231</v>
+      <c r="A80" s="13"/>
+      <c r="B80" s="13"/>
+      <c r="C80" s="13"/>
+      <c r="D80" s="13"/>
+      <c r="E80" s="13"/>
+      <c r="F80" s="13"/>
+      <c r="G80" s="13"/>
+      <c r="H80" s="13"/>
+      <c r="I80" s="13"/>
+      <c r="J80" s="13"/>
+      <c r="K80" s="4" t="s">
+        <v>226</v>
       </c>
       <c r="L80" s="2"/>
       <c r="M80" s="2"/>
@@ -7827,18 +7848,32 @@
       <c r="AA80" s="2"/>
     </row>
     <row r="81" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="10"/>
-      <c r="B81" s="10"/>
-      <c r="C81" s="10"/>
-      <c r="D81" s="10"/>
-      <c r="E81" s="10"/>
-      <c r="F81" s="10"/>
-      <c r="G81" s="10"/>
-      <c r="H81" s="10"/>
-      <c r="I81" s="10"/>
-      <c r="J81" s="10"/>
+      <c r="A81" s="14" t="s">
+        <v>227</v>
+      </c>
+      <c r="B81" s="12" t="s">
+        <v>228</v>
+      </c>
+      <c r="C81" s="19" t="s">
+        <v>229</v>
+      </c>
+      <c r="D81" s="12">
+        <v>44</v>
+      </c>
+      <c r="E81" s="12">
+        <v>3709</v>
+      </c>
+      <c r="F81" s="12" t="s">
+        <v>230</v>
+      </c>
+      <c r="G81" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H81" s="12"/>
+      <c r="I81" s="12"/>
+      <c r="J81" s="12"/>
       <c r="K81" s="3" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="L81" s="2"/>
       <c r="M81" s="2"/>
@@ -7858,18 +7893,18 @@
       <c r="AA81" s="2"/>
     </row>
     <row r="82" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="10"/>
-      <c r="B82" s="10"/>
-      <c r="C82" s="10"/>
-      <c r="D82" s="10"/>
-      <c r="E82" s="10"/>
-      <c r="F82" s="10"/>
-      <c r="G82" s="10"/>
-      <c r="H82" s="10"/>
-      <c r="I82" s="10"/>
-      <c r="J82" s="10"/>
+      <c r="A82" s="15"/>
+      <c r="B82" s="15"/>
+      <c r="C82" s="15"/>
+      <c r="D82" s="15"/>
+      <c r="E82" s="15"/>
+      <c r="F82" s="15"/>
+      <c r="G82" s="15"/>
+      <c r="H82" s="15"/>
+      <c r="I82" s="15"/>
+      <c r="J82" s="15"/>
       <c r="K82" s="3" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="L82" s="2"/>
       <c r="M82" s="2"/>
@@ -7889,18 +7924,18 @@
       <c r="AA82" s="2"/>
     </row>
     <row r="83" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="11"/>
-      <c r="B83" s="11"/>
-      <c r="C83" s="11"/>
-      <c r="D83" s="11"/>
-      <c r="E83" s="11"/>
-      <c r="F83" s="11"/>
-      <c r="G83" s="11"/>
-      <c r="H83" s="11"/>
-      <c r="I83" s="11"/>
-      <c r="J83" s="11"/>
-      <c r="K83" s="4" t="s">
-        <v>234</v>
+      <c r="A83" s="15"/>
+      <c r="B83" s="15"/>
+      <c r="C83" s="15"/>
+      <c r="D83" s="15"/>
+      <c r="E83" s="15"/>
+      <c r="F83" s="15"/>
+      <c r="G83" s="15"/>
+      <c r="H83" s="15"/>
+      <c r="I83" s="15"/>
+      <c r="J83" s="15"/>
+      <c r="K83" s="3" t="s">
+        <v>233</v>
       </c>
       <c r="L83" s="2"/>
       <c r="M83" s="2"/>
@@ -7920,34 +7955,18 @@
       <c r="AA83" s="2"/>
     </row>
     <row r="84" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="12" t="s">
-        <v>235</v>
-      </c>
-      <c r="B84" s="9" t="s">
-        <v>236</v>
-      </c>
-      <c r="C84" s="16" t="s">
-        <v>237</v>
-      </c>
-      <c r="D84" s="4">
-        <v>1122</v>
-      </c>
-      <c r="E84" s="4">
-        <v>157909</v>
-      </c>
-      <c r="F84" s="4" t="s">
-        <v>238</v>
-      </c>
-      <c r="G84" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="H84" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="I84" s="4"/>
-      <c r="J84" s="4"/>
-      <c r="K84" s="3" t="s">
-        <v>239</v>
+      <c r="A84" s="13"/>
+      <c r="B84" s="13"/>
+      <c r="C84" s="13"/>
+      <c r="D84" s="13"/>
+      <c r="E84" s="13"/>
+      <c r="F84" s="13"/>
+      <c r="G84" s="13"/>
+      <c r="H84" s="13"/>
+      <c r="I84" s="13"/>
+      <c r="J84" s="13"/>
+      <c r="K84" s="4" t="s">
+        <v>234</v>
       </c>
       <c r="L84" s="2"/>
       <c r="M84" s="2"/>
@@ -7967,17 +7986,23 @@
       <c r="AA84" s="2"/>
     </row>
     <row r="85" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="10"/>
-      <c r="B85" s="10"/>
-      <c r="C85" s="17"/>
+      <c r="A85" s="14" t="s">
+        <v>235</v>
+      </c>
+      <c r="B85" s="12" t="s">
+        <v>236</v>
+      </c>
+      <c r="C85" s="16" t="s">
+        <v>237</v>
+      </c>
       <c r="D85" s="4">
-        <v>263</v>
+        <v>1122</v>
       </c>
       <c r="E85" s="4">
-        <v>26260</v>
-      </c>
-      <c r="F85" s="7" t="s">
-        <v>240</v>
+        <v>157909</v>
+      </c>
+      <c r="F85" s="4" t="s">
+        <v>238</v>
       </c>
       <c r="G85" s="4" t="s">
         <v>16</v>
@@ -7988,7 +8013,7 @@
       <c r="I85" s="4"/>
       <c r="J85" s="4"/>
       <c r="K85" s="3" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="L85" s="2"/>
       <c r="M85" s="2"/>
@@ -8008,14 +8033,14 @@
       <c r="AA85" s="2"/>
     </row>
     <row r="86" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="10"/>
-      <c r="B86" s="10"/>
+      <c r="A86" s="15"/>
+      <c r="B86" s="15"/>
       <c r="C86" s="17"/>
       <c r="D86" s="4">
-        <v>144</v>
+        <v>263</v>
       </c>
       <c r="E86" s="4">
-        <v>16293</v>
+        <v>26260</v>
       </c>
       <c r="F86" s="7" t="s">
         <v>240</v>
@@ -8029,7 +8054,7 @@
       <c r="I86" s="4"/>
       <c r="J86" s="4"/>
       <c r="K86" s="3" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="L86" s="2"/>
       <c r="M86" s="2"/>
@@ -8049,24 +8074,28 @@
       <c r="AA86" s="2"/>
     </row>
     <row r="87" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A87" s="11"/>
-      <c r="B87" s="11"/>
-      <c r="C87" s="18"/>
+      <c r="A87" s="15"/>
+      <c r="B87" s="15"/>
+      <c r="C87" s="17"/>
       <c r="D87" s="4">
-        <v>254</v>
+        <v>144</v>
       </c>
       <c r="E87" s="4">
-        <v>15469</v>
+        <v>16293</v>
       </c>
       <c r="F87" s="7" t="s">
         <v>240</v>
       </c>
-      <c r="G87" s="4"/>
-      <c r="H87" s="4"/>
+      <c r="G87" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H87" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="I87" s="4"/>
       <c r="J87" s="4"/>
-      <c r="K87" s="4" t="s">
-        <v>243</v>
+      <c r="K87" s="3" t="s">
+        <v>242</v>
       </c>
       <c r="L87" s="2"/>
       <c r="M87" s="2"/>
@@ -8086,26 +8115,24 @@
       <c r="AA87" s="2"/>
     </row>
     <row r="88" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A88" s="5" t="s">
-        <v>244</v>
-      </c>
-      <c r="B88" s="4" t="s">
-        <v>245</v>
-      </c>
-      <c r="C88" s="6" t="s">
-        <v>246</v>
-      </c>
-      <c r="D88" s="4"/>
-      <c r="E88" s="4"/>
-      <c r="F88" s="4" t="s">
-        <v>247</v>
+      <c r="A88" s="13"/>
+      <c r="B88" s="13"/>
+      <c r="C88" s="18"/>
+      <c r="D88" s="4">
+        <v>254</v>
+      </c>
+      <c r="E88" s="4">
+        <v>15469</v>
+      </c>
+      <c r="F88" s="7" t="s">
+        <v>240</v>
       </c>
       <c r="G88" s="4"/>
       <c r="H88" s="4"/>
       <c r="I88" s="4"/>
       <c r="J88" s="4"/>
       <c r="K88" s="4" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="L88" s="2"/>
       <c r="M88" s="2"/>
@@ -8126,24 +8153,26 @@
     </row>
     <row r="89" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="5" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="B89" s="4" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="C89" s="6" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="D89" s="4"/>
       <c r="E89" s="4"/>
       <c r="F89" s="4" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="G89" s="4"/>
       <c r="H89" s="4"/>
       <c r="I89" s="4"/>
       <c r="J89" s="4"/>
-      <c r="K89" s="4"/>
+      <c r="K89" s="4" t="s">
+        <v>248</v>
+      </c>
       <c r="L89" s="2"/>
       <c r="M89" s="2"/>
       <c r="N89" s="2"/>
@@ -8163,18 +8192,18 @@
     </row>
     <row r="90" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="5" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="B90" s="4" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="C90" s="6" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="D90" s="4"/>
       <c r="E90" s="4"/>
       <c r="F90" s="4" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="G90" s="4"/>
       <c r="H90" s="4"/>
@@ -8200,26 +8229,24 @@
     </row>
     <row r="91" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="5" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="B91" s="4" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="C91" s="6" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
       <c r="D91" s="4"/>
       <c r="E91" s="4"/>
       <c r="F91" s="4" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="G91" s="4"/>
       <c r="H91" s="4"/>
       <c r="I91" s="4"/>
       <c r="J91" s="4"/>
-      <c r="K91" s="4" t="s">
-        <v>261</v>
-      </c>
+      <c r="K91" s="4"/>
       <c r="L91" s="2"/>
       <c r="M91" s="2"/>
       <c r="N91" s="2"/>
@@ -8239,25 +8266,25 @@
     </row>
     <row r="92" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="5" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="B92" s="4" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="C92" s="6" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="D92" s="4"/>
       <c r="E92" s="4"/>
       <c r="F92" s="4" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="G92" s="4"/>
       <c r="H92" s="4"/>
       <c r="I92" s="4"/>
       <c r="J92" s="4"/>
       <c r="K92" s="4" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="L92" s="2"/>
       <c r="M92" s="2"/>
@@ -8278,24 +8305,26 @@
     </row>
     <row r="93" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="5" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="B93" s="4" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="C93" s="6" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="D93" s="4"/>
       <c r="E93" s="4"/>
       <c r="F93" s="4" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="G93" s="4"/>
       <c r="H93" s="4"/>
       <c r="I93" s="4"/>
       <c r="J93" s="4"/>
-      <c r="K93" s="4"/>
+      <c r="K93" s="4" t="s">
+        <v>266</v>
+      </c>
       <c r="L93" s="2"/>
       <c r="M93" s="2"/>
       <c r="N93" s="2"/>
@@ -8315,18 +8344,18 @@
     </row>
     <row r="94" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="5" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="B94" s="4" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="C94" s="6" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="D94" s="4"/>
       <c r="E94" s="4"/>
       <c r="F94" s="4" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="G94" s="4"/>
       <c r="H94" s="4"/>
@@ -8352,26 +8381,24 @@
     </row>
     <row r="95" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="5" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="B95" s="4" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="C95" s="6" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="D95" s="4"/>
       <c r="E95" s="4"/>
       <c r="F95" s="4" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="G95" s="4"/>
       <c r="H95" s="4"/>
       <c r="I95" s="4"/>
       <c r="J95" s="4"/>
-      <c r="K95" s="4" t="s">
-        <v>266</v>
-      </c>
+      <c r="K95" s="4"/>
       <c r="L95" s="2"/>
       <c r="M95" s="2"/>
       <c r="N95" s="2"/>
@@ -8391,24 +8418,26 @@
     </row>
     <row r="96" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="5" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="B96" s="4" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="C96" s="6" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="D96" s="4"/>
       <c r="E96" s="4"/>
       <c r="F96" s="4" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="G96" s="4"/>
       <c r="H96" s="4"/>
       <c r="I96" s="4"/>
       <c r="J96" s="4"/>
-      <c r="K96" s="4"/>
+      <c r="K96" s="4" t="s">
+        <v>266</v>
+      </c>
       <c r="L96" s="2"/>
       <c r="M96" s="2"/>
       <c r="N96" s="2"/>
@@ -8428,26 +8457,24 @@
     </row>
     <row r="97" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="5" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="B97" s="4" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="C97" s="6" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="D97" s="4"/>
       <c r="E97" s="4"/>
       <c r="F97" s="4" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="G97" s="4"/>
       <c r="H97" s="4"/>
       <c r="I97" s="4"/>
       <c r="J97" s="4"/>
-      <c r="K97" s="4" t="s">
-        <v>287</v>
-      </c>
+      <c r="K97" s="4"/>
       <c r="L97" s="2"/>
       <c r="M97" s="2"/>
       <c r="N97" s="2"/>
@@ -8467,25 +8494,25 @@
     </row>
     <row r="98" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="5" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="B98" s="4" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
       <c r="C98" s="6" t="s">
-        <v>290</v>
+        <v>285</v>
       </c>
       <c r="D98" s="4"/>
       <c r="E98" s="4"/>
       <c r="F98" s="4" t="s">
-        <v>291</v>
+        <v>286</v>
       </c>
       <c r="G98" s="4"/>
       <c r="H98" s="4"/>
       <c r="I98" s="4"/>
       <c r="J98" s="4"/>
       <c r="K98" s="4" t="s">
-        <v>292</v>
+        <v>287</v>
       </c>
       <c r="L98" s="2"/>
       <c r="M98" s="2"/>
@@ -8506,24 +8533,26 @@
     </row>
     <row r="99" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="5" t="s">
-        <v>293</v>
+        <v>288</v>
       </c>
       <c r="B99" s="4" t="s">
-        <v>294</v>
+        <v>289</v>
       </c>
       <c r="C99" s="6" t="s">
-        <v>295</v>
+        <v>290</v>
       </c>
       <c r="D99" s="4"/>
       <c r="E99" s="4"/>
       <c r="F99" s="4" t="s">
-        <v>296</v>
+        <v>291</v>
       </c>
       <c r="G99" s="4"/>
       <c r="H99" s="4"/>
       <c r="I99" s="4"/>
       <c r="J99" s="4"/>
-      <c r="K99" s="4"/>
+      <c r="K99" s="4" t="s">
+        <v>292</v>
+      </c>
       <c r="L99" s="2"/>
       <c r="M99" s="2"/>
       <c r="N99" s="2"/>
@@ -8543,26 +8572,24 @@
     </row>
     <row r="100" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="5" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="B100" s="4" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="C100" s="6" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="D100" s="4"/>
       <c r="E100" s="4"/>
       <c r="F100" s="4" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="G100" s="4"/>
       <c r="H100" s="4"/>
       <c r="I100" s="4"/>
       <c r="J100" s="4"/>
-      <c r="K100" s="4" t="s">
-        <v>292</v>
-      </c>
+      <c r="K100" s="4"/>
       <c r="L100" s="2"/>
       <c r="M100" s="2"/>
       <c r="N100" s="2"/>
@@ -8582,24 +8609,26 @@
     </row>
     <row r="101" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="5" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="B101" s="4" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
       <c r="C101" s="6" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
       <c r="D101" s="4"/>
       <c r="E101" s="4"/>
       <c r="F101" s="4" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="G101" s="4"/>
       <c r="H101" s="4"/>
       <c r="I101" s="4"/>
       <c r="J101" s="4"/>
-      <c r="K101" s="4"/>
+      <c r="K101" s="4" t="s">
+        <v>292</v>
+      </c>
       <c r="L101" s="2"/>
       <c r="M101" s="2"/>
       <c r="N101" s="2"/>
@@ -8619,18 +8648,18 @@
     </row>
     <row r="102" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A102" s="5" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="B102" s="4" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="C102" s="6" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="D102" s="4"/>
       <c r="E102" s="4"/>
       <c r="F102" s="4" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="G102" s="4"/>
       <c r="H102" s="4"/>
@@ -8656,18 +8685,18 @@
     </row>
     <row r="103" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="5" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
       <c r="B103" s="4" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
       <c r="C103" s="6" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="D103" s="4"/>
       <c r="E103" s="4"/>
       <c r="F103" s="4" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="G103" s="4"/>
       <c r="H103" s="4"/>
@@ -8693,18 +8722,18 @@
     </row>
     <row r="104" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="5" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="B104" s="4" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="C104" s="6" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="D104" s="4"/>
       <c r="E104" s="4"/>
       <c r="F104" s="4" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="G104" s="4"/>
       <c r="H104" s="4"/>
@@ -8730,26 +8759,24 @@
     </row>
     <row r="105" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="5" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="B105" s="4" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="C105" s="6" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="D105" s="4"/>
       <c r="E105" s="4"/>
       <c r="F105" s="4" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="G105" s="4"/>
       <c r="H105" s="4"/>
       <c r="I105" s="4"/>
       <c r="J105" s="4"/>
-      <c r="K105" s="4" t="s">
-        <v>292</v>
-      </c>
+      <c r="K105" s="4"/>
       <c r="L105" s="2"/>
       <c r="M105" s="2"/>
       <c r="N105" s="2"/>
@@ -8769,24 +8796,26 @@
     </row>
     <row r="106" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A106" s="5" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="B106" s="4" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="C106" s="6" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="D106" s="4"/>
       <c r="E106" s="4"/>
       <c r="F106" s="4" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="G106" s="4"/>
       <c r="H106" s="4"/>
       <c r="I106" s="4"/>
       <c r="J106" s="4"/>
-      <c r="K106" s="4"/>
+      <c r="K106" s="4" t="s">
+        <v>292</v>
+      </c>
       <c r="L106" s="2"/>
       <c r="M106" s="2"/>
       <c r="N106" s="2"/>
@@ -8806,18 +8835,18 @@
     </row>
     <row r="107" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" s="5" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="B107" s="4" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="C107" s="6" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="D107" s="4"/>
       <c r="E107" s="4"/>
       <c r="F107" s="4" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="G107" s="4"/>
       <c r="H107" s="4"/>
@@ -8843,18 +8872,18 @@
     </row>
     <row r="108" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108" s="5" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="B108" s="4" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="C108" s="6" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="D108" s="4"/>
       <c r="E108" s="4"/>
       <c r="F108" s="4" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="G108" s="4"/>
       <c r="H108" s="4"/>
@@ -8880,18 +8909,18 @@
     </row>
     <row r="109" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A109" s="5" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="B109" s="4" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
       <c r="C109" s="6" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
       <c r="D109" s="4"/>
       <c r="E109" s="4"/>
       <c r="F109" s="4" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="G109" s="4"/>
       <c r="H109" s="4"/>
@@ -8917,18 +8946,18 @@
     </row>
     <row r="110" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110" s="5" t="s">
-        <v>337</v>
+        <v>333</v>
       </c>
       <c r="B110" s="4" t="s">
-        <v>338</v>
+        <v>334</v>
       </c>
       <c r="C110" s="6" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
       <c r="D110" s="4"/>
       <c r="E110" s="4"/>
       <c r="F110" s="4" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
       <c r="G110" s="4"/>
       <c r="H110" s="4"/>
@@ -8954,26 +8983,24 @@
     </row>
     <row r="111" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A111" s="5" t="s">
-        <v>341</v>
+        <v>337</v>
       </c>
       <c r="B111" s="4" t="s">
-        <v>342</v>
+        <v>338</v>
       </c>
       <c r="C111" s="6" t="s">
-        <v>343</v>
+        <v>339</v>
       </c>
       <c r="D111" s="4"/>
       <c r="E111" s="4"/>
       <c r="F111" s="4" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
       <c r="G111" s="4"/>
       <c r="H111" s="4"/>
       <c r="I111" s="4"/>
       <c r="J111" s="4"/>
-      <c r="K111" s="4" t="s">
-        <v>345</v>
-      </c>
+      <c r="K111" s="4"/>
       <c r="L111" s="2"/>
       <c r="M111" s="2"/>
       <c r="N111" s="2"/>
@@ -8993,24 +9020,26 @@
     </row>
     <row r="112" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A112" s="5" t="s">
-        <v>346</v>
+        <v>341</v>
       </c>
       <c r="B112" s="4" t="s">
-        <v>347</v>
+        <v>342</v>
       </c>
       <c r="C112" s="6" t="s">
-        <v>348</v>
+        <v>343</v>
       </c>
       <c r="D112" s="4"/>
       <c r="E112" s="4"/>
       <c r="F112" s="4" t="s">
-        <v>349</v>
+        <v>344</v>
       </c>
       <c r="G112" s="4"/>
       <c r="H112" s="4"/>
       <c r="I112" s="4"/>
       <c r="J112" s="4"/>
-      <c r="K112" s="4"/>
+      <c r="K112" s="4" t="s">
+        <v>345</v>
+      </c>
       <c r="L112" s="2"/>
       <c r="M112" s="2"/>
       <c r="N112" s="2"/>
@@ -9030,26 +9059,24 @@
     </row>
     <row r="113" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A113" s="5" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="B113" s="4" t="s">
-        <v>351</v>
+        <v>347</v>
       </c>
       <c r="C113" s="6" t="s">
-        <v>352</v>
+        <v>348</v>
       </c>
       <c r="D113" s="4"/>
       <c r="E113" s="4"/>
       <c r="F113" s="4" t="s">
-        <v>353</v>
+        <v>349</v>
       </c>
       <c r="G113" s="4"/>
       <c r="H113" s="4"/>
       <c r="I113" s="4"/>
       <c r="J113" s="4"/>
-      <c r="K113" s="4" t="s">
-        <v>354</v>
-      </c>
+      <c r="K113" s="4"/>
       <c r="L113" s="2"/>
       <c r="M113" s="2"/>
       <c r="N113" s="2"/>
@@ -9069,24 +9096,26 @@
     </row>
     <row r="114" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A114" s="5" t="s">
-        <v>355</v>
+        <v>350</v>
       </c>
       <c r="B114" s="4" t="s">
-        <v>356</v>
+        <v>351</v>
       </c>
       <c r="C114" s="6" t="s">
-        <v>357</v>
+        <v>352</v>
       </c>
       <c r="D114" s="4"/>
       <c r="E114" s="4"/>
       <c r="F114" s="4" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
       <c r="G114" s="4"/>
       <c r="H114" s="4"/>
       <c r="I114" s="4"/>
       <c r="J114" s="4"/>
-      <c r="K114" s="4"/>
+      <c r="K114" s="4" t="s">
+        <v>354</v>
+      </c>
       <c r="L114" s="2"/>
       <c r="M114" s="2"/>
       <c r="N114" s="2"/>
@@ -9106,18 +9135,18 @@
     </row>
     <row r="115" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A115" s="5" t="s">
-        <v>359</v>
+        <v>355</v>
       </c>
       <c r="B115" s="4" t="s">
-        <v>360</v>
+        <v>356</v>
       </c>
       <c r="C115" s="6" t="s">
-        <v>361</v>
+        <v>357</v>
       </c>
       <c r="D115" s="4"/>
       <c r="E115" s="4"/>
       <c r="F115" s="4" t="s">
-        <v>362</v>
+        <v>358</v>
       </c>
       <c r="G115" s="4"/>
       <c r="H115" s="4"/>
@@ -9143,18 +9172,18 @@
     </row>
     <row r="116" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116" s="5" t="s">
-        <v>363</v>
+        <v>359</v>
       </c>
       <c r="B116" s="4" t="s">
-        <v>364</v>
+        <v>360</v>
       </c>
       <c r="C116" s="6" t="s">
-        <v>365</v>
+        <v>361</v>
       </c>
       <c r="D116" s="4"/>
       <c r="E116" s="4"/>
       <c r="F116" s="4" t="s">
-        <v>366</v>
+        <v>362</v>
       </c>
       <c r="G116" s="4"/>
       <c r="H116" s="4"/>
@@ -9180,18 +9209,18 @@
     </row>
     <row r="117" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="B117" s="4" t="s">
-        <v>368</v>
+        <v>364</v>
       </c>
       <c r="C117" s="6" t="s">
-        <v>369</v>
+        <v>365</v>
       </c>
       <c r="D117" s="4"/>
       <c r="E117" s="4"/>
       <c r="F117" s="4" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="G117" s="4"/>
       <c r="H117" s="4"/>
@@ -9215,28 +9244,26 @@
       <c r="Z117" s="2"/>
       <c r="AA117" s="2"/>
     </row>
-    <row r="118" spans="1:27" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A118" s="12" t="s">
-        <v>371</v>
-      </c>
-      <c r="B118" s="9" t="s">
-        <v>372</v>
-      </c>
-      <c r="C118" s="13" t="s">
-        <v>373</v>
-      </c>
-      <c r="D118" s="9"/>
-      <c r="E118" s="9"/>
-      <c r="F118" s="9" t="s">
-        <v>374</v>
-      </c>
-      <c r="G118" s="9"/>
-      <c r="H118" s="9"/>
-      <c r="I118" s="9"/>
-      <c r="J118" s="9"/>
-      <c r="K118" s="3" t="s">
-        <v>375</v>
-      </c>
+    <row r="118" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A118" s="5" t="s">
+        <v>367</v>
+      </c>
+      <c r="B118" s="4" t="s">
+        <v>368</v>
+      </c>
+      <c r="C118" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="D118" s="4"/>
+      <c r="E118" s="4"/>
+      <c r="F118" s="4" t="s">
+        <v>370</v>
+      </c>
+      <c r="G118" s="4"/>
+      <c r="H118" s="4"/>
+      <c r="I118" s="4"/>
+      <c r="J118" s="4"/>
+      <c r="K118" s="4"/>
       <c r="L118" s="2"/>
       <c r="M118" s="2"/>
       <c r="N118" s="2"/>
@@ -9254,19 +9281,27 @@
       <c r="Z118" s="2"/>
       <c r="AA118" s="2"/>
     </row>
-    <row r="119" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A119" s="11"/>
-      <c r="B119" s="11"/>
-      <c r="C119" s="11"/>
-      <c r="D119" s="11"/>
-      <c r="E119" s="11"/>
-      <c r="F119" s="11"/>
-      <c r="G119" s="11"/>
-      <c r="H119" s="11"/>
-      <c r="I119" s="11"/>
-      <c r="J119" s="11"/>
-      <c r="K119" s="4" t="s">
-        <v>376</v>
+    <row r="119" spans="1:27" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A119" s="14" t="s">
+        <v>371</v>
+      </c>
+      <c r="B119" s="12" t="s">
+        <v>372</v>
+      </c>
+      <c r="C119" s="19" t="s">
+        <v>373</v>
+      </c>
+      <c r="D119" s="12"/>
+      <c r="E119" s="12"/>
+      <c r="F119" s="12" t="s">
+        <v>374</v>
+      </c>
+      <c r="G119" s="12"/>
+      <c r="H119" s="12"/>
+      <c r="I119" s="12"/>
+      <c r="J119" s="12"/>
+      <c r="K119" s="3" t="s">
+        <v>375</v>
       </c>
       <c r="L119" s="2"/>
       <c r="M119" s="2"/>
@@ -9286,25 +9321,19 @@
       <c r="AA119" s="2"/>
     </row>
     <row r="120" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A120" s="5" t="s">
-        <v>377</v>
-      </c>
-      <c r="B120" s="4" t="s">
-        <v>378</v>
-      </c>
-      <c r="C120" s="6" t="s">
-        <v>379</v>
-      </c>
-      <c r="D120" s="4"/>
-      <c r="E120" s="4"/>
-      <c r="F120" s="4" t="s">
-        <v>380</v>
-      </c>
-      <c r="G120" s="4"/>
-      <c r="H120" s="4"/>
-      <c r="I120" s="4"/>
-      <c r="J120" s="4"/>
-      <c r="K120" s="4"/>
+      <c r="A120" s="13"/>
+      <c r="B120" s="13"/>
+      <c r="C120" s="13"/>
+      <c r="D120" s="13"/>
+      <c r="E120" s="13"/>
+      <c r="F120" s="13"/>
+      <c r="G120" s="13"/>
+      <c r="H120" s="13"/>
+      <c r="I120" s="13"/>
+      <c r="J120" s="13"/>
+      <c r="K120" s="4" t="s">
+        <v>376</v>
+      </c>
       <c r="L120" s="2"/>
       <c r="M120" s="2"/>
       <c r="N120" s="2"/>
@@ -9324,26 +9353,24 @@
     </row>
     <row r="121" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A121" s="5" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
       <c r="B121" s="4" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
       <c r="C121" s="6" t="s">
-        <v>383</v>
+        <v>379</v>
       </c>
       <c r="D121" s="4"/>
       <c r="E121" s="4"/>
       <c r="F121" s="4" t="s">
-        <v>384</v>
+        <v>380</v>
       </c>
       <c r="G121" s="4"/>
       <c r="H121" s="4"/>
       <c r="I121" s="4"/>
       <c r="J121" s="4"/>
-      <c r="K121" s="4" t="s">
-        <v>385</v>
-      </c>
+      <c r="K121" s="4"/>
       <c r="L121" s="2"/>
       <c r="M121" s="2"/>
       <c r="N121" s="2"/>
@@ -9363,24 +9390,26 @@
     </row>
     <row r="122" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A122" s="5" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="B122" s="4" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
       <c r="C122" s="6" t="s">
-        <v>388</v>
+        <v>383</v>
       </c>
       <c r="D122" s="4"/>
       <c r="E122" s="4"/>
       <c r="F122" s="4" t="s">
-        <v>389</v>
+        <v>384</v>
       </c>
       <c r="G122" s="4"/>
       <c r="H122" s="4"/>
       <c r="I122" s="4"/>
       <c r="J122" s="4"/>
-      <c r="K122" s="4"/>
+      <c r="K122" s="4" t="s">
+        <v>385</v>
+      </c>
       <c r="L122" s="2"/>
       <c r="M122" s="2"/>
       <c r="N122" s="2"/>
@@ -9400,18 +9429,18 @@
     </row>
     <row r="123" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A123" s="5" t="s">
-        <v>390</v>
+        <v>386</v>
       </c>
       <c r="B123" s="4" t="s">
-        <v>391</v>
+        <v>387</v>
       </c>
       <c r="C123" s="6" t="s">
-        <v>392</v>
+        <v>388</v>
       </c>
       <c r="D123" s="4"/>
       <c r="E123" s="4"/>
       <c r="F123" s="4" t="s">
-        <v>393</v>
+        <v>389</v>
       </c>
       <c r="G123" s="4"/>
       <c r="H123" s="4"/>
@@ -9437,18 +9466,18 @@
     </row>
     <row r="124" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A124" s="5" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
       <c r="B124" s="4" t="s">
-        <v>395</v>
+        <v>391</v>
       </c>
       <c r="C124" s="6" t="s">
-        <v>396</v>
+        <v>392</v>
       </c>
       <c r="D124" s="4"/>
       <c r="E124" s="4"/>
       <c r="F124" s="4" t="s">
-        <v>397</v>
+        <v>393</v>
       </c>
       <c r="G124" s="4"/>
       <c r="H124" s="4"/>
@@ -9474,26 +9503,24 @@
     </row>
     <row r="125" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A125" s="5" t="s">
-        <v>398</v>
+        <v>394</v>
       </c>
       <c r="B125" s="4" t="s">
-        <v>399</v>
+        <v>395</v>
       </c>
       <c r="C125" s="6" t="s">
-        <v>400</v>
+        <v>396</v>
       </c>
       <c r="D125" s="4"/>
       <c r="E125" s="4"/>
       <c r="F125" s="4" t="s">
-        <v>401</v>
+        <v>397</v>
       </c>
       <c r="G125" s="4"/>
       <c r="H125" s="4"/>
       <c r="I125" s="4"/>
       <c r="J125" s="4"/>
-      <c r="K125" s="4" t="s">
-        <v>402</v>
-      </c>
+      <c r="K125" s="4"/>
       <c r="L125" s="2"/>
       <c r="M125" s="2"/>
       <c r="N125" s="2"/>
@@ -9513,24 +9540,26 @@
     </row>
     <row r="126" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A126" s="5" t="s">
-        <v>403</v>
+        <v>398</v>
       </c>
       <c r="B126" s="4" t="s">
-        <v>404</v>
+        <v>399</v>
       </c>
       <c r="C126" s="6" t="s">
-        <v>405</v>
+        <v>400</v>
       </c>
       <c r="D126" s="4"/>
       <c r="E126" s="4"/>
       <c r="F126" s="4" t="s">
-        <v>406</v>
+        <v>401</v>
       </c>
       <c r="G126" s="4"/>
       <c r="H126" s="4"/>
       <c r="I126" s="4"/>
       <c r="J126" s="4"/>
-      <c r="K126" s="4"/>
+      <c r="K126" s="4" t="s">
+        <v>402</v>
+      </c>
       <c r="L126" s="2"/>
       <c r="M126" s="2"/>
       <c r="N126" s="2"/>
@@ -9550,18 +9579,18 @@
     </row>
     <row r="127" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A127" s="5" t="s">
-        <v>407</v>
+        <v>403</v>
       </c>
       <c r="B127" s="4" t="s">
-        <v>408</v>
+        <v>404</v>
       </c>
       <c r="C127" s="6" t="s">
-        <v>409</v>
+        <v>405</v>
       </c>
       <c r="D127" s="4"/>
       <c r="E127" s="4"/>
       <c r="F127" s="4" t="s">
-        <v>410</v>
+        <v>406</v>
       </c>
       <c r="G127" s="4"/>
       <c r="H127" s="4"/>
@@ -9587,18 +9616,18 @@
     </row>
     <row r="128" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A128" s="5" t="s">
-        <v>411</v>
+        <v>407</v>
       </c>
       <c r="B128" s="4" t="s">
-        <v>412</v>
+        <v>408</v>
       </c>
       <c r="C128" s="6" t="s">
-        <v>413</v>
+        <v>409</v>
       </c>
       <c r="D128" s="4"/>
       <c r="E128" s="4"/>
       <c r="F128" s="4" t="s">
-        <v>414</v>
+        <v>410</v>
       </c>
       <c r="G128" s="4"/>
       <c r="H128" s="4"/>
@@ -9624,18 +9653,18 @@
     </row>
     <row r="129" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A129" s="5" t="s">
-        <v>415</v>
+        <v>411</v>
       </c>
       <c r="B129" s="4" t="s">
-        <v>416</v>
+        <v>412</v>
       </c>
       <c r="C129" s="6" t="s">
-        <v>417</v>
+        <v>413</v>
       </c>
       <c r="D129" s="4"/>
       <c r="E129" s="4"/>
       <c r="F129" s="4" t="s">
-        <v>418</v>
+        <v>414</v>
       </c>
       <c r="G129" s="4"/>
       <c r="H129" s="4"/>
@@ -9661,18 +9690,18 @@
     </row>
     <row r="130" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A130" s="5" t="s">
-        <v>419</v>
+        <v>415</v>
       </c>
       <c r="B130" s="4" t="s">
-        <v>420</v>
+        <v>416</v>
       </c>
       <c r="C130" s="6" t="s">
-        <v>421</v>
+        <v>417</v>
       </c>
       <c r="D130" s="4"/>
       <c r="E130" s="4"/>
       <c r="F130" s="4" t="s">
-        <v>422</v>
+        <v>418</v>
       </c>
       <c r="G130" s="4"/>
       <c r="H130" s="4"/>
@@ -9698,18 +9727,18 @@
     </row>
     <row r="131" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A131" s="5" t="s">
-        <v>423</v>
+        <v>419</v>
       </c>
       <c r="B131" s="4" t="s">
-        <v>424</v>
+        <v>420</v>
       </c>
       <c r="C131" s="6" t="s">
-        <v>425</v>
+        <v>421</v>
       </c>
       <c r="D131" s="4"/>
       <c r="E131" s="4"/>
       <c r="F131" s="4" t="s">
-        <v>426</v>
+        <v>422</v>
       </c>
       <c r="G131" s="4"/>
       <c r="H131" s="4"/>
@@ -9735,18 +9764,18 @@
     </row>
     <row r="132" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A132" s="5" t="s">
-        <v>427</v>
+        <v>423</v>
       </c>
       <c r="B132" s="4" t="s">
-        <v>428</v>
+        <v>424</v>
       </c>
       <c r="C132" s="6" t="s">
-        <v>429</v>
+        <v>425</v>
       </c>
       <c r="D132" s="4"/>
       <c r="E132" s="4"/>
       <c r="F132" s="4" t="s">
-        <v>430</v>
+        <v>426</v>
       </c>
       <c r="G132" s="4"/>
       <c r="H132" s="4"/>
@@ -9772,18 +9801,18 @@
     </row>
     <row r="133" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A133" s="5" t="s">
-        <v>431</v>
+        <v>427</v>
       </c>
       <c r="B133" s="4" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
       <c r="C133" s="6" t="s">
-        <v>433</v>
+        <v>429</v>
       </c>
       <c r="D133" s="4"/>
       <c r="E133" s="4"/>
       <c r="F133" s="4" t="s">
-        <v>434</v>
+        <v>430</v>
       </c>
       <c r="G133" s="4"/>
       <c r="H133" s="4"/>
@@ -9809,18 +9838,18 @@
     </row>
     <row r="134" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A134" s="5" t="s">
-        <v>435</v>
+        <v>431</v>
       </c>
       <c r="B134" s="4" t="s">
-        <v>436</v>
+        <v>432</v>
       </c>
       <c r="C134" s="6" t="s">
-        <v>437</v>
+        <v>433</v>
       </c>
       <c r="D134" s="4"/>
       <c r="E134" s="4"/>
       <c r="F134" s="4" t="s">
-        <v>438</v>
+        <v>434</v>
       </c>
       <c r="G134" s="4"/>
       <c r="H134" s="4"/>
@@ -9846,18 +9875,18 @@
     </row>
     <row r="135" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A135" s="5" t="s">
-        <v>439</v>
+        <v>435</v>
       </c>
       <c r="B135" s="4" t="s">
-        <v>440</v>
+        <v>436</v>
       </c>
       <c r="C135" s="6" t="s">
-        <v>441</v>
+        <v>437</v>
       </c>
       <c r="D135" s="4"/>
       <c r="E135" s="4"/>
       <c r="F135" s="4" t="s">
-        <v>442</v>
+        <v>438</v>
       </c>
       <c r="G135" s="4"/>
       <c r="H135" s="4"/>
@@ -9883,18 +9912,18 @@
     </row>
     <row r="136" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A136" s="5" t="s">
-        <v>443</v>
+        <v>439</v>
       </c>
       <c r="B136" s="4" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="C136" s="6" t="s">
-        <v>445</v>
+        <v>441</v>
       </c>
       <c r="D136" s="4"/>
       <c r="E136" s="4"/>
       <c r="F136" s="4" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="G136" s="4"/>
       <c r="H136" s="4"/>
@@ -9920,18 +9949,18 @@
     </row>
     <row r="137" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A137" s="5" t="s">
-        <v>447</v>
+        <v>443</v>
       </c>
       <c r="B137" s="4" t="s">
-        <v>448</v>
+        <v>444</v>
       </c>
       <c r="C137" s="6" t="s">
-        <v>449</v>
+        <v>445</v>
       </c>
       <c r="D137" s="4"/>
       <c r="E137" s="4"/>
       <c r="F137" s="4" t="s">
-        <v>450</v>
+        <v>446</v>
       </c>
       <c r="G137" s="4"/>
       <c r="H137" s="4"/>
@@ -9957,18 +9986,18 @@
     </row>
     <row r="138" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A138" s="5" t="s">
-        <v>451</v>
+        <v>447</v>
       </c>
       <c r="B138" s="4" t="s">
-        <v>452</v>
+        <v>448</v>
       </c>
       <c r="C138" s="6" t="s">
-        <v>453</v>
+        <v>449</v>
       </c>
       <c r="D138" s="4"/>
       <c r="E138" s="4"/>
       <c r="F138" s="4" t="s">
-        <v>454</v>
+        <v>450</v>
       </c>
       <c r="G138" s="4"/>
       <c r="H138" s="4"/>
@@ -9994,18 +10023,18 @@
     </row>
     <row r="139" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A139" s="5" t="s">
-        <v>455</v>
+        <v>451</v>
       </c>
       <c r="B139" s="4" t="s">
-        <v>456</v>
+        <v>452</v>
       </c>
       <c r="C139" s="6" t="s">
-        <v>457</v>
+        <v>453</v>
       </c>
       <c r="D139" s="4"/>
       <c r="E139" s="4"/>
       <c r="F139" s="4" t="s">
-        <v>458</v>
+        <v>454</v>
       </c>
       <c r="G139" s="4"/>
       <c r="H139" s="4"/>
@@ -10031,18 +10060,18 @@
     </row>
     <row r="140" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A140" s="5" t="s">
-        <v>459</v>
+        <v>455</v>
       </c>
       <c r="B140" s="4" t="s">
-        <v>460</v>
+        <v>456</v>
       </c>
       <c r="C140" s="6" t="s">
-        <v>461</v>
+        <v>457</v>
       </c>
       <c r="D140" s="4"/>
       <c r="E140" s="4"/>
       <c r="F140" s="4" t="s">
-        <v>462</v>
+        <v>458</v>
       </c>
       <c r="G140" s="4"/>
       <c r="H140" s="4"/>
@@ -10068,18 +10097,18 @@
     </row>
     <row r="141" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A141" s="5" t="s">
-        <v>463</v>
+        <v>459</v>
       </c>
       <c r="B141" s="4" t="s">
-        <v>464</v>
+        <v>460</v>
       </c>
       <c r="C141" s="6" t="s">
-        <v>465</v>
+        <v>461</v>
       </c>
       <c r="D141" s="4"/>
       <c r="E141" s="4"/>
       <c r="F141" s="4" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
       <c r="G141" s="4"/>
       <c r="H141" s="4"/>
@@ -10105,18 +10134,18 @@
     </row>
     <row r="142" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A142" s="5" t="s">
-        <v>467</v>
+        <v>463</v>
       </c>
       <c r="B142" s="4" t="s">
-        <v>468</v>
+        <v>464</v>
       </c>
       <c r="C142" s="6" t="s">
-        <v>469</v>
+        <v>465</v>
       </c>
       <c r="D142" s="4"/>
       <c r="E142" s="4"/>
       <c r="F142" s="4" t="s">
-        <v>470</v>
+        <v>466</v>
       </c>
       <c r="G142" s="4"/>
       <c r="H142" s="4"/>
@@ -10142,18 +10171,18 @@
     </row>
     <row r="143" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A143" s="5" t="s">
-        <v>471</v>
+        <v>467</v>
       </c>
       <c r="B143" s="4" t="s">
-        <v>472</v>
+        <v>468</v>
       </c>
       <c r="C143" s="6" t="s">
-        <v>473</v>
+        <v>469</v>
       </c>
       <c r="D143" s="4"/>
       <c r="E143" s="4"/>
       <c r="F143" s="4" t="s">
-        <v>474</v>
+        <v>470</v>
       </c>
       <c r="G143" s="4"/>
       <c r="H143" s="4"/>
@@ -10179,18 +10208,18 @@
     </row>
     <row r="144" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A144" s="5" t="s">
-        <v>475</v>
+        <v>471</v>
       </c>
       <c r="B144" s="4" t="s">
-        <v>476</v>
+        <v>472</v>
       </c>
       <c r="C144" s="6" t="s">
-        <v>477</v>
+        <v>473</v>
       </c>
       <c r="D144" s="4"/>
       <c r="E144" s="4"/>
       <c r="F144" s="4" t="s">
-        <v>478</v>
+        <v>474</v>
       </c>
       <c r="G144" s="4"/>
       <c r="H144" s="4"/>
@@ -10216,18 +10245,18 @@
     </row>
     <row r="145" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A145" s="5" t="s">
-        <v>479</v>
+        <v>475</v>
       </c>
       <c r="B145" s="4" t="s">
-        <v>480</v>
+        <v>476</v>
       </c>
       <c r="C145" s="6" t="s">
-        <v>481</v>
+        <v>477</v>
       </c>
       <c r="D145" s="4"/>
       <c r="E145" s="4"/>
       <c r="F145" s="4" t="s">
-        <v>482</v>
+        <v>478</v>
       </c>
       <c r="G145" s="4"/>
       <c r="H145" s="4"/>
@@ -10253,18 +10282,18 @@
     </row>
     <row r="146" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A146" s="5" t="s">
-        <v>483</v>
+        <v>479</v>
       </c>
       <c r="B146" s="4" t="s">
-        <v>484</v>
+        <v>480</v>
       </c>
       <c r="C146" s="6" t="s">
-        <v>485</v>
+        <v>481</v>
       </c>
       <c r="D146" s="4"/>
       <c r="E146" s="4"/>
       <c r="F146" s="4" t="s">
-        <v>486</v>
+        <v>482</v>
       </c>
       <c r="G146" s="4"/>
       <c r="H146" s="4"/>
@@ -10290,16 +10319,18 @@
     </row>
     <row r="147" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A147" s="5" t="s">
-        <v>487</v>
+        <v>483</v>
       </c>
       <c r="B147" s="4" t="s">
-        <v>488</v>
-      </c>
-      <c r="C147" s="6"/>
+        <v>484</v>
+      </c>
+      <c r="C147" s="6" t="s">
+        <v>485</v>
+      </c>
       <c r="D147" s="4"/>
       <c r="E147" s="4"/>
       <c r="F147" s="4" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="G147" s="4"/>
       <c r="H147" s="4"/>
@@ -10325,16 +10356,16 @@
     </row>
     <row r="148" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A148" s="5" t="s">
-        <v>490</v>
+        <v>487</v>
       </c>
       <c r="B148" s="4" t="s">
-        <v>491</v>
+        <v>488</v>
       </c>
       <c r="C148" s="6"/>
       <c r="D148" s="4"/>
       <c r="E148" s="4"/>
       <c r="F148" s="4" t="s">
-        <v>492</v>
+        <v>489</v>
       </c>
       <c r="G148" s="4"/>
       <c r="H148" s="4"/>
@@ -10360,16 +10391,16 @@
     </row>
     <row r="149" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A149" s="5" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
       <c r="B149" s="4" t="s">
-        <v>494</v>
+        <v>491</v>
       </c>
       <c r="C149" s="6"/>
       <c r="D149" s="4"/>
       <c r="E149" s="4"/>
       <c r="F149" s="4" t="s">
-        <v>495</v>
+        <v>492</v>
       </c>
       <c r="G149" s="4"/>
       <c r="H149" s="4"/>
@@ -10395,16 +10426,16 @@
     </row>
     <row r="150" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A150" s="5" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="B150" s="4" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
       <c r="C150" s="6"/>
       <c r="D150" s="4"/>
       <c r="E150" s="4"/>
       <c r="F150" s="4" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
       <c r="G150" s="4"/>
       <c r="H150" s="4"/>
@@ -10430,16 +10461,16 @@
     </row>
     <row r="151" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A151" s="5" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
       <c r="B151" s="4" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
       <c r="C151" s="6"/>
       <c r="D151" s="4"/>
       <c r="E151" s="4"/>
       <c r="F151" s="4" t="s">
-        <v>501</v>
+        <v>498</v>
       </c>
       <c r="G151" s="4"/>
       <c r="H151" s="4"/>
@@ -10465,16 +10496,16 @@
     </row>
     <row r="152" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A152" s="5" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
       <c r="B152" s="4" t="s">
-        <v>503</v>
+        <v>500</v>
       </c>
       <c r="C152" s="6"/>
       <c r="D152" s="4"/>
       <c r="E152" s="4"/>
       <c r="F152" s="4" t="s">
-        <v>504</v>
+        <v>501</v>
       </c>
       <c r="G152" s="4"/>
       <c r="H152" s="4"/>
@@ -10500,16 +10531,16 @@
     </row>
     <row r="153" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A153" s="5" t="s">
-        <v>505</v>
+        <v>502</v>
       </c>
       <c r="B153" s="4" t="s">
-        <v>506</v>
+        <v>503</v>
       </c>
       <c r="C153" s="6"/>
       <c r="D153" s="4"/>
       <c r="E153" s="4"/>
       <c r="F153" s="4" t="s">
-        <v>507</v>
+        <v>504</v>
       </c>
       <c r="G153" s="4"/>
       <c r="H153" s="4"/>
@@ -10535,16 +10566,16 @@
     </row>
     <row r="154" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A154" s="5" t="s">
-        <v>508</v>
+        <v>505</v>
       </c>
       <c r="B154" s="4" t="s">
-        <v>509</v>
+        <v>506</v>
       </c>
       <c r="C154" s="6"/>
       <c r="D154" s="4"/>
       <c r="E154" s="4"/>
       <c r="F154" s="4" t="s">
-        <v>510</v>
+        <v>507</v>
       </c>
       <c r="G154" s="4"/>
       <c r="H154" s="4"/>
@@ -10570,16 +10601,16 @@
     </row>
     <row r="155" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A155" s="5" t="s">
-        <v>511</v>
+        <v>508</v>
       </c>
       <c r="B155" s="4" t="s">
-        <v>512</v>
+        <v>509</v>
       </c>
       <c r="C155" s="6"/>
       <c r="D155" s="4"/>
       <c r="E155" s="4"/>
       <c r="F155" s="4" t="s">
-        <v>513</v>
+        <v>510</v>
       </c>
       <c r="G155" s="4"/>
       <c r="H155" s="4"/>
@@ -10604,17 +10635,23 @@
       <c r="AA155" s="2"/>
     </row>
     <row r="156" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A156" s="2"/>
-      <c r="B156" s="2"/>
-      <c r="C156" s="8"/>
-      <c r="D156" s="2"/>
-      <c r="E156" s="2"/>
-      <c r="F156" s="2"/>
-      <c r="G156" s="2"/>
-      <c r="H156" s="2"/>
-      <c r="I156" s="2"/>
-      <c r="J156" s="2"/>
-      <c r="K156" s="2"/>
+      <c r="A156" s="5" t="s">
+        <v>511</v>
+      </c>
+      <c r="B156" s="4" t="s">
+        <v>512</v>
+      </c>
+      <c r="C156" s="6"/>
+      <c r="D156" s="4"/>
+      <c r="E156" s="4"/>
+      <c r="F156" s="4" t="s">
+        <v>513</v>
+      </c>
+      <c r="G156" s="4"/>
+      <c r="H156" s="4"/>
+      <c r="I156" s="4"/>
+      <c r="J156" s="4"/>
+      <c r="K156" s="4"/>
       <c r="L156" s="2"/>
       <c r="M156" s="2"/>
       <c r="N156" s="2"/>
@@ -35137,21 +35174,97 @@
       <c r="Z1001" s="2"/>
       <c r="AA1001" s="2"/>
     </row>
+    <row r="1002" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1002" s="2"/>
+      <c r="B1002" s="2"/>
+      <c r="C1002" s="8"/>
+      <c r="D1002" s="2"/>
+      <c r="E1002" s="2"/>
+      <c r="F1002" s="2"/>
+      <c r="G1002" s="2"/>
+      <c r="H1002" s="2"/>
+      <c r="I1002" s="2"/>
+      <c r="J1002" s="2"/>
+      <c r="K1002" s="2"/>
+      <c r="L1002" s="2"/>
+      <c r="M1002" s="2"/>
+      <c r="N1002" s="2"/>
+      <c r="O1002" s="2"/>
+      <c r="P1002" s="2"/>
+      <c r="Q1002" s="2"/>
+      <c r="R1002" s="2"/>
+      <c r="S1002" s="2"/>
+      <c r="T1002" s="2"/>
+      <c r="U1002" s="2"/>
+      <c r="V1002" s="2"/>
+      <c r="W1002" s="2"/>
+      <c r="X1002" s="2"/>
+      <c r="Y1002" s="2"/>
+      <c r="Z1002" s="2"/>
+      <c r="AA1002" s="2"/>
+    </row>
   </sheetData>
   <mergeCells count="84">
-    <mergeCell ref="J118:J119"/>
-    <mergeCell ref="A84:A87"/>
-    <mergeCell ref="B84:B87"/>
-    <mergeCell ref="C84:C87"/>
-    <mergeCell ref="A118:A119"/>
-    <mergeCell ref="B118:B119"/>
-    <mergeCell ref="C118:C119"/>
-    <mergeCell ref="D118:D119"/>
-    <mergeCell ref="E118:E119"/>
-    <mergeCell ref="F118:F119"/>
-    <mergeCell ref="G118:G119"/>
-    <mergeCell ref="H118:H119"/>
-    <mergeCell ref="I118:I119"/>
+    <mergeCell ref="H35:H38"/>
+    <mergeCell ref="I35:I38"/>
+    <mergeCell ref="J35:J38"/>
+    <mergeCell ref="A35:A38"/>
+    <mergeCell ref="B35:B38"/>
+    <mergeCell ref="C35:C38"/>
+    <mergeCell ref="D35:D38"/>
+    <mergeCell ref="E35:E38"/>
+    <mergeCell ref="F35:F38"/>
+    <mergeCell ref="G35:G38"/>
+    <mergeCell ref="H45:H71"/>
+    <mergeCell ref="I45:I71"/>
+    <mergeCell ref="J45:J71"/>
+    <mergeCell ref="A45:A71"/>
+    <mergeCell ref="B45:B71"/>
+    <mergeCell ref="C45:C71"/>
+    <mergeCell ref="D45:D71"/>
+    <mergeCell ref="E45:E71"/>
+    <mergeCell ref="F45:F71"/>
+    <mergeCell ref="G45:G71"/>
+    <mergeCell ref="H76:H80"/>
+    <mergeCell ref="I76:I80"/>
+    <mergeCell ref="J76:J80"/>
+    <mergeCell ref="A76:A80"/>
+    <mergeCell ref="B76:B80"/>
+    <mergeCell ref="C76:C80"/>
+    <mergeCell ref="D76:D80"/>
+    <mergeCell ref="E76:E80"/>
+    <mergeCell ref="F76:F80"/>
+    <mergeCell ref="G76:G80"/>
+    <mergeCell ref="H81:H84"/>
+    <mergeCell ref="I81:I84"/>
+    <mergeCell ref="J81:J84"/>
+    <mergeCell ref="A81:A84"/>
+    <mergeCell ref="B81:B84"/>
+    <mergeCell ref="C81:C84"/>
+    <mergeCell ref="D81:D84"/>
+    <mergeCell ref="E81:E84"/>
+    <mergeCell ref="F81:F84"/>
+    <mergeCell ref="G81:G84"/>
+    <mergeCell ref="I1:I3"/>
+    <mergeCell ref="J1:J3"/>
+    <mergeCell ref="K1:K3"/>
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="B1:B3"/>
+    <mergeCell ref="C1:C3"/>
+    <mergeCell ref="D1:D3"/>
+    <mergeCell ref="E1:E3"/>
+    <mergeCell ref="G1:G3"/>
+    <mergeCell ref="H1:H3"/>
+    <mergeCell ref="H16:H17"/>
+    <mergeCell ref="I16:I17"/>
+    <mergeCell ref="J16:J17"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="D16:D17"/>
+    <mergeCell ref="E16:E17"/>
+    <mergeCell ref="F16:F17"/>
+    <mergeCell ref="G16:G17"/>
     <mergeCell ref="H20:H21"/>
     <mergeCell ref="I20:I21"/>
     <mergeCell ref="J20:J21"/>
@@ -35163,66 +35276,19 @@
     <mergeCell ref="E20:E21"/>
     <mergeCell ref="F20:F21"/>
     <mergeCell ref="G20:G21"/>
-    <mergeCell ref="H16:H17"/>
-    <mergeCell ref="I16:I17"/>
-    <mergeCell ref="J16:J17"/>
-    <mergeCell ref="A16:A17"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="D16:D17"/>
-    <mergeCell ref="E16:E17"/>
-    <mergeCell ref="F16:F17"/>
-    <mergeCell ref="G16:G17"/>
-    <mergeCell ref="I1:I3"/>
-    <mergeCell ref="J1:J3"/>
-    <mergeCell ref="K1:K3"/>
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="B1:B3"/>
-    <mergeCell ref="C1:C3"/>
-    <mergeCell ref="D1:D3"/>
-    <mergeCell ref="E1:E3"/>
-    <mergeCell ref="G1:G3"/>
-    <mergeCell ref="H1:H3"/>
-    <mergeCell ref="H80:H83"/>
-    <mergeCell ref="I80:I83"/>
-    <mergeCell ref="J80:J83"/>
-    <mergeCell ref="A80:A83"/>
-    <mergeCell ref="B80:B83"/>
-    <mergeCell ref="C80:C83"/>
-    <mergeCell ref="D80:D83"/>
-    <mergeCell ref="E80:E83"/>
-    <mergeCell ref="F80:F83"/>
-    <mergeCell ref="G80:G83"/>
-    <mergeCell ref="H75:H79"/>
-    <mergeCell ref="I75:I79"/>
-    <mergeCell ref="J75:J79"/>
-    <mergeCell ref="A75:A79"/>
-    <mergeCell ref="B75:B79"/>
-    <mergeCell ref="C75:C79"/>
-    <mergeCell ref="D75:D79"/>
-    <mergeCell ref="E75:E79"/>
-    <mergeCell ref="F75:F79"/>
-    <mergeCell ref="G75:G79"/>
-    <mergeCell ref="H45:H71"/>
-    <mergeCell ref="I45:I71"/>
-    <mergeCell ref="J45:J71"/>
-    <mergeCell ref="A45:A71"/>
-    <mergeCell ref="B45:B71"/>
-    <mergeCell ref="C45:C71"/>
-    <mergeCell ref="D45:D71"/>
-    <mergeCell ref="E45:E71"/>
-    <mergeCell ref="F45:F71"/>
-    <mergeCell ref="G45:G71"/>
-    <mergeCell ref="H35:H38"/>
-    <mergeCell ref="I35:I38"/>
-    <mergeCell ref="J35:J38"/>
-    <mergeCell ref="A35:A38"/>
-    <mergeCell ref="B35:B38"/>
-    <mergeCell ref="C35:C38"/>
-    <mergeCell ref="D35:D38"/>
-    <mergeCell ref="E35:E38"/>
-    <mergeCell ref="F35:F38"/>
-    <mergeCell ref="G35:G38"/>
+    <mergeCell ref="J119:J120"/>
+    <mergeCell ref="A85:A88"/>
+    <mergeCell ref="B85:B88"/>
+    <mergeCell ref="C85:C88"/>
+    <mergeCell ref="A119:A120"/>
+    <mergeCell ref="B119:B120"/>
+    <mergeCell ref="C119:C120"/>
+    <mergeCell ref="D119:D120"/>
+    <mergeCell ref="E119:E120"/>
+    <mergeCell ref="F119:F120"/>
+    <mergeCell ref="G119:G120"/>
+    <mergeCell ref="H119:H120"/>
+    <mergeCell ref="I119:I120"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="portrait"/>

</xml_diff>

<commit_message>
updated files for the Battle of uhud
</commit_message>
<xml_diff>
--- a/data/meta/Witness_list_sheet.xlsx
+++ b/data/meta/Witness_list_sheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rkjin\github\Sirah-Project\data\meta\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70504173-9427-4472-9CD7-B0986782F42A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B42618E-28E4-4834-8F8E-FB83DC8F8AEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="624" uniqueCount="522">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="628" uniqueCount="526">
   <si>
     <t>Arabic name</t>
   </si>
@@ -4257,6 +4257,18 @@
   </si>
   <si>
     <t xml:space="preserve">8/05/26 Name added to directory. Not added to github as of this date. </t>
+  </si>
+  <si>
+    <t>Nūḥ b. Abī Maryam</t>
+  </si>
+  <si>
+    <t>WNIAM</t>
+  </si>
+  <si>
+    <t>ابن أبي مريم</t>
+  </si>
+  <si>
+    <t>added 08/11/26</t>
   </si>
 </sst>
 </file>
@@ -4454,19 +4466,23 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
@@ -4476,15 +4492,11 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4700,7 +4712,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AA1002"/>
+  <dimension ref="A1:AA1003"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.140625" customWidth="1"/>
@@ -4716,16 +4728,16 @@
   <sheetData>
     <row r="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A1" s="21"/>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="15" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="15" t="s">
         <v>3</v>
       </c>
       <c r="F1" s="1" t="s">
@@ -4740,10 +4752,10 @@
       <c r="I1" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="12" t="s">
+      <c r="J1" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="12" t="s">
+      <c r="K1" s="15" t="s">
         <v>9</v>
       </c>
       <c r="L1" s="2"/>
@@ -4764,19 +4776,19 @@
       <c r="AA1" s="2"/>
     </row>
     <row r="2" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A2" s="15"/>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
+      <c r="A2" s="16"/>
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
       <c r="F2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
-      <c r="I2" s="15"/>
-      <c r="J2" s="15"/>
-      <c r="K2" s="15"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
+      <c r="I2" s="16"/>
+      <c r="J2" s="16"/>
+      <c r="K2" s="16"/>
       <c r="L2" s="2"/>
       <c r="M2" s="2"/>
       <c r="N2" s="2"/>
@@ -4795,19 +4807,19 @@
       <c r="AA2" s="2"/>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A3" s="13"/>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
+      <c r="A3" s="17"/>
+      <c r="B3" s="17"/>
+      <c r="C3" s="17"/>
+      <c r="D3" s="17"/>
+      <c r="E3" s="17"/>
       <c r="F3" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="G3" s="13"/>
-      <c r="H3" s="13"/>
-      <c r="I3" s="13"/>
-      <c r="J3" s="13"/>
-      <c r="K3" s="13"/>
+      <c r="G3" s="17"/>
+      <c r="H3" s="17"/>
+      <c r="I3" s="17"/>
+      <c r="J3" s="17"/>
+      <c r="K3" s="17"/>
       <c r="L3" s="2"/>
       <c r="M3" s="2"/>
       <c r="N3" s="2"/>
@@ -5390,32 +5402,32 @@
       <c r="AA15" s="2"/>
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A16" s="14" t="s">
+      <c r="A16" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="B16" s="12" t="s">
+      <c r="B16" s="15" t="s">
         <v>69</v>
       </c>
       <c r="C16" s="19" t="s">
         <v>70</v>
       </c>
-      <c r="D16" s="12">
+      <c r="D16" s="15">
         <v>2</v>
       </c>
-      <c r="E16" s="12">
+      <c r="E16" s="15">
         <v>223</v>
       </c>
-      <c r="F16" s="12" t="s">
+      <c r="F16" s="15" t="s">
         <v>71</v>
       </c>
-      <c r="G16" s="12" t="s">
+      <c r="G16" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="H16" s="12" t="s">
+      <c r="H16" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="I16" s="12"/>
-      <c r="J16" s="12"/>
+      <c r="I16" s="15"/>
+      <c r="J16" s="15"/>
       <c r="K16" s="3" t="s">
         <v>72</v>
       </c>
@@ -5437,16 +5449,16 @@
       <c r="AA16" s="2"/>
     </row>
     <row r="17" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A17" s="13"/>
-      <c r="B17" s="13"/>
-      <c r="C17" s="13"/>
-      <c r="D17" s="13"/>
-      <c r="E17" s="13"/>
-      <c r="F17" s="13"/>
-      <c r="G17" s="13"/>
-      <c r="H17" s="13"/>
-      <c r="I17" s="13"/>
-      <c r="J17" s="13"/>
+      <c r="A17" s="17"/>
+      <c r="B17" s="17"/>
+      <c r="C17" s="17"/>
+      <c r="D17" s="17"/>
+      <c r="E17" s="17"/>
+      <c r="F17" s="17"/>
+      <c r="G17" s="17"/>
+      <c r="H17" s="17"/>
+      <c r="I17" s="17"/>
+      <c r="J17" s="17"/>
       <c r="K17" s="4" t="s">
         <v>73</v>
       </c>
@@ -5562,33 +5574,33 @@
       <c r="AA19" s="2"/>
     </row>
     <row r="20" spans="1:27" ht="108" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="14" t="s">
+      <c r="A20" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="B20" s="12" t="s">
+      <c r="B20" s="15" t="s">
         <v>84</v>
       </c>
       <c r="C20" s="19" t="s">
         <v>85</v>
       </c>
-      <c r="D20" s="12">
+      <c r="D20" s="15">
         <v>12</v>
       </c>
-      <c r="E20" s="12">
+      <c r="E20" s="15">
         <v>1427</v>
       </c>
-      <c r="F20" s="12" t="s">
+      <c r="F20" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="G20" s="12" t="s">
+      <c r="G20" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="H20" s="12" t="s">
+      <c r="H20" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="I20" s="12"/>
-      <c r="J20" s="12"/>
-      <c r="K20" s="12" t="s">
+      <c r="I20" s="15"/>
+      <c r="J20" s="15"/>
+      <c r="K20" s="15" t="s">
         <v>82</v>
       </c>
       <c r="L20" s="2"/>
@@ -5609,17 +5621,17 @@
       <c r="AA20" s="2"/>
     </row>
     <row r="21" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="13"/>
-      <c r="B21" s="13"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="13"/>
-      <c r="E21" s="13"/>
-      <c r="F21" s="13"/>
-      <c r="G21" s="13"/>
-      <c r="H21" s="13"/>
-      <c r="I21" s="13"/>
-      <c r="J21" s="13"/>
-      <c r="K21" s="13"/>
+      <c r="A21" s="17"/>
+      <c r="B21" s="17"/>
+      <c r="C21" s="17"/>
+      <c r="D21" s="17"/>
+      <c r="E21" s="17"/>
+      <c r="F21" s="17"/>
+      <c r="G21" s="17"/>
+      <c r="H21" s="17"/>
+      <c r="I21" s="17"/>
+      <c r="J21" s="17"/>
+      <c r="K21" s="17"/>
       <c r="L21" s="2"/>
       <c r="M21" s="2"/>
       <c r="N21" s="2"/>
@@ -6239,32 +6251,32 @@
       <c r="AA34" s="2"/>
     </row>
     <row r="35" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="14" t="s">
+      <c r="A35" s="18" t="s">
         <v>145</v>
       </c>
-      <c r="B35" s="12" t="s">
+      <c r="B35" s="15" t="s">
         <v>146</v>
       </c>
       <c r="C35" s="19" t="s">
         <v>147</v>
       </c>
-      <c r="D35" s="12">
+      <c r="D35" s="15">
         <v>44</v>
       </c>
-      <c r="E35" s="12">
+      <c r="E35" s="15">
         <v>3981</v>
       </c>
-      <c r="F35" s="12" t="s">
+      <c r="F35" s="15" t="s">
         <v>148</v>
       </c>
-      <c r="G35" s="12" t="s">
+      <c r="G35" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="H35" s="12" t="s">
+      <c r="H35" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="I35" s="12"/>
-      <c r="J35" s="12"/>
+      <c r="I35" s="15"/>
+      <c r="J35" s="15"/>
       <c r="K35" s="3" t="s">
         <v>149</v>
       </c>
@@ -6286,16 +6298,16 @@
       <c r="AA35" s="2"/>
     </row>
     <row r="36" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="15"/>
-      <c r="B36" s="15"/>
-      <c r="C36" s="15"/>
-      <c r="D36" s="15"/>
-      <c r="E36" s="15"/>
-      <c r="F36" s="15"/>
-      <c r="G36" s="15"/>
-      <c r="H36" s="15"/>
-      <c r="I36" s="15"/>
-      <c r="J36" s="15"/>
+      <c r="A36" s="16"/>
+      <c r="B36" s="16"/>
+      <c r="C36" s="16"/>
+      <c r="D36" s="16"/>
+      <c r="E36" s="16"/>
+      <c r="F36" s="16"/>
+      <c r="G36" s="16"/>
+      <c r="H36" s="16"/>
+      <c r="I36" s="16"/>
+      <c r="J36" s="16"/>
       <c r="K36" s="3" t="s">
         <v>150</v>
       </c>
@@ -6317,16 +6329,16 @@
       <c r="AA36" s="2"/>
     </row>
     <row r="37" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="15"/>
-      <c r="B37" s="15"/>
-      <c r="C37" s="15"/>
-      <c r="D37" s="15"/>
-      <c r="E37" s="15"/>
-      <c r="F37" s="15"/>
-      <c r="G37" s="15"/>
-      <c r="H37" s="15"/>
-      <c r="I37" s="15"/>
-      <c r="J37" s="15"/>
+      <c r="A37" s="16"/>
+      <c r="B37" s="16"/>
+      <c r="C37" s="16"/>
+      <c r="D37" s="16"/>
+      <c r="E37" s="16"/>
+      <c r="F37" s="16"/>
+      <c r="G37" s="16"/>
+      <c r="H37" s="16"/>
+      <c r="I37" s="16"/>
+      <c r="J37" s="16"/>
       <c r="K37" s="3"/>
       <c r="L37" s="2"/>
       <c r="M37" s="2"/>
@@ -6346,16 +6358,16 @@
       <c r="AA37" s="2"/>
     </row>
     <row r="38" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="13"/>
-      <c r="B38" s="13"/>
-      <c r="C38" s="13"/>
-      <c r="D38" s="13"/>
-      <c r="E38" s="13"/>
-      <c r="F38" s="13"/>
-      <c r="G38" s="13"/>
-      <c r="H38" s="13"/>
-      <c r="I38" s="13"/>
-      <c r="J38" s="13"/>
+      <c r="A38" s="17"/>
+      <c r="B38" s="17"/>
+      <c r="C38" s="17"/>
+      <c r="D38" s="17"/>
+      <c r="E38" s="17"/>
+      <c r="F38" s="17"/>
+      <c r="G38" s="17"/>
+      <c r="H38" s="17"/>
+      <c r="I38" s="17"/>
+      <c r="J38" s="17"/>
       <c r="K38" s="4" t="s">
         <v>151</v>
       </c>
@@ -6653,28 +6665,28 @@
       <c r="AA44" s="2"/>
     </row>
     <row r="45" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="14" t="s">
+      <c r="A45" s="18" t="s">
         <v>179</v>
       </c>
-      <c r="B45" s="12" t="s">
+      <c r="B45" s="15" t="s">
         <v>180</v>
       </c>
       <c r="C45" s="19" t="s">
         <v>181</v>
       </c>
-      <c r="D45" s="12">
+      <c r="D45" s="15">
         <v>48</v>
       </c>
-      <c r="E45" s="12">
+      <c r="E45" s="15">
         <v>10207</v>
       </c>
-      <c r="F45" s="12" t="s">
+      <c r="F45" s="15" t="s">
         <v>182</v>
       </c>
-      <c r="G45" s="12"/>
-      <c r="H45" s="12"/>
-      <c r="I45" s="12"/>
-      <c r="J45" s="12"/>
+      <c r="G45" s="15"/>
+      <c r="H45" s="15"/>
+      <c r="I45" s="15"/>
+      <c r="J45" s="15"/>
       <c r="K45" s="3" t="s">
         <v>183</v>
       </c>
@@ -6696,16 +6708,16 @@
       <c r="AA45" s="2"/>
     </row>
     <row r="46" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="15"/>
-      <c r="B46" s="15"/>
-      <c r="C46" s="15"/>
-      <c r="D46" s="15"/>
-      <c r="E46" s="15"/>
-      <c r="F46" s="15"/>
-      <c r="G46" s="15"/>
-      <c r="H46" s="15"/>
-      <c r="I46" s="15"/>
-      <c r="J46" s="15"/>
+      <c r="A46" s="16"/>
+      <c r="B46" s="16"/>
+      <c r="C46" s="16"/>
+      <c r="D46" s="16"/>
+      <c r="E46" s="16"/>
+      <c r="F46" s="16"/>
+      <c r="G46" s="16"/>
+      <c r="H46" s="16"/>
+      <c r="I46" s="16"/>
+      <c r="J46" s="16"/>
       <c r="K46" s="3" t="s">
         <v>184</v>
       </c>
@@ -6727,16 +6739,16 @@
       <c r="AA46" s="2"/>
     </row>
     <row r="47" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="15"/>
-      <c r="B47" s="15"/>
-      <c r="C47" s="15"/>
-      <c r="D47" s="15"/>
-      <c r="E47" s="15"/>
-      <c r="F47" s="15"/>
-      <c r="G47" s="15"/>
-      <c r="H47" s="15"/>
-      <c r="I47" s="15"/>
-      <c r="J47" s="15"/>
+      <c r="A47" s="16"/>
+      <c r="B47" s="16"/>
+      <c r="C47" s="16"/>
+      <c r="D47" s="16"/>
+      <c r="E47" s="16"/>
+      <c r="F47" s="16"/>
+      <c r="G47" s="16"/>
+      <c r="H47" s="16"/>
+      <c r="I47" s="16"/>
+      <c r="J47" s="16"/>
       <c r="K47" s="3" t="s">
         <v>185</v>
       </c>
@@ -6758,16 +6770,16 @@
       <c r="AA47" s="2"/>
     </row>
     <row r="48" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="15"/>
-      <c r="B48" s="15"/>
-      <c r="C48" s="15"/>
-      <c r="D48" s="15"/>
-      <c r="E48" s="15"/>
-      <c r="F48" s="15"/>
-      <c r="G48" s="15"/>
-      <c r="H48" s="15"/>
-      <c r="I48" s="15"/>
-      <c r="J48" s="15"/>
+      <c r="A48" s="16"/>
+      <c r="B48" s="16"/>
+      <c r="C48" s="16"/>
+      <c r="D48" s="16"/>
+      <c r="E48" s="16"/>
+      <c r="F48" s="16"/>
+      <c r="G48" s="16"/>
+      <c r="H48" s="16"/>
+      <c r="I48" s="16"/>
+      <c r="J48" s="16"/>
       <c r="K48" s="3" t="s">
         <v>186</v>
       </c>
@@ -6789,16 +6801,16 @@
       <c r="AA48" s="2"/>
     </row>
     <row r="49" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="15"/>
-      <c r="B49" s="15"/>
-      <c r="C49" s="15"/>
-      <c r="D49" s="15"/>
-      <c r="E49" s="15"/>
-      <c r="F49" s="15"/>
-      <c r="G49" s="15"/>
-      <c r="H49" s="15"/>
-      <c r="I49" s="15"/>
-      <c r="J49" s="15"/>
+      <c r="A49" s="16"/>
+      <c r="B49" s="16"/>
+      <c r="C49" s="16"/>
+      <c r="D49" s="16"/>
+      <c r="E49" s="16"/>
+      <c r="F49" s="16"/>
+      <c r="G49" s="16"/>
+      <c r="H49" s="16"/>
+      <c r="I49" s="16"/>
+      <c r="J49" s="16"/>
       <c r="K49" s="3" t="s">
         <v>187</v>
       </c>
@@ -6820,16 +6832,16 @@
       <c r="AA49" s="2"/>
     </row>
     <row r="50" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="15"/>
-      <c r="B50" s="15"/>
-      <c r="C50" s="15"/>
-      <c r="D50" s="15"/>
-      <c r="E50" s="15"/>
-      <c r="F50" s="15"/>
-      <c r="G50" s="15"/>
-      <c r="H50" s="15"/>
-      <c r="I50" s="15"/>
-      <c r="J50" s="15"/>
+      <c r="A50" s="16"/>
+      <c r="B50" s="16"/>
+      <c r="C50" s="16"/>
+      <c r="D50" s="16"/>
+      <c r="E50" s="16"/>
+      <c r="F50" s="16"/>
+      <c r="G50" s="16"/>
+      <c r="H50" s="16"/>
+      <c r="I50" s="16"/>
+      <c r="J50" s="16"/>
       <c r="K50" s="3" t="s">
         <v>188</v>
       </c>
@@ -6851,16 +6863,16 @@
       <c r="AA50" s="2"/>
     </row>
     <row r="51" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="15"/>
-      <c r="B51" s="15"/>
-      <c r="C51" s="15"/>
-      <c r="D51" s="15"/>
-      <c r="E51" s="15"/>
-      <c r="F51" s="15"/>
-      <c r="G51" s="15"/>
-      <c r="H51" s="15"/>
-      <c r="I51" s="15"/>
-      <c r="J51" s="15"/>
+      <c r="A51" s="16"/>
+      <c r="B51" s="16"/>
+      <c r="C51" s="16"/>
+      <c r="D51" s="16"/>
+      <c r="E51" s="16"/>
+      <c r="F51" s="16"/>
+      <c r="G51" s="16"/>
+      <c r="H51" s="16"/>
+      <c r="I51" s="16"/>
+      <c r="J51" s="16"/>
       <c r="K51" s="3" t="s">
         <v>189</v>
       </c>
@@ -6882,16 +6894,16 @@
       <c r="AA51" s="2"/>
     </row>
     <row r="52" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="15"/>
-      <c r="B52" s="15"/>
-      <c r="C52" s="15"/>
-      <c r="D52" s="15"/>
-      <c r="E52" s="15"/>
-      <c r="F52" s="15"/>
-      <c r="G52" s="15"/>
-      <c r="H52" s="15"/>
-      <c r="I52" s="15"/>
-      <c r="J52" s="15"/>
+      <c r="A52" s="16"/>
+      <c r="B52" s="16"/>
+      <c r="C52" s="16"/>
+      <c r="D52" s="16"/>
+      <c r="E52" s="16"/>
+      <c r="F52" s="16"/>
+      <c r="G52" s="16"/>
+      <c r="H52" s="16"/>
+      <c r="I52" s="16"/>
+      <c r="J52" s="16"/>
       <c r="K52" s="3" t="s">
         <v>190</v>
       </c>
@@ -6913,16 +6925,16 @@
       <c r="AA52" s="2"/>
     </row>
     <row r="53" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="15"/>
-      <c r="B53" s="15"/>
-      <c r="C53" s="15"/>
-      <c r="D53" s="15"/>
-      <c r="E53" s="15"/>
-      <c r="F53" s="15"/>
-      <c r="G53" s="15"/>
-      <c r="H53" s="15"/>
-      <c r="I53" s="15"/>
-      <c r="J53" s="15"/>
+      <c r="A53" s="16"/>
+      <c r="B53" s="16"/>
+      <c r="C53" s="16"/>
+      <c r="D53" s="16"/>
+      <c r="E53" s="16"/>
+      <c r="F53" s="16"/>
+      <c r="G53" s="16"/>
+      <c r="H53" s="16"/>
+      <c r="I53" s="16"/>
+      <c r="J53" s="16"/>
       <c r="K53" s="3" t="s">
         <v>191</v>
       </c>
@@ -6944,16 +6956,16 @@
       <c r="AA53" s="2"/>
     </row>
     <row r="54" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="15"/>
-      <c r="B54" s="15"/>
-      <c r="C54" s="15"/>
-      <c r="D54" s="15"/>
-      <c r="E54" s="15"/>
-      <c r="F54" s="15"/>
-      <c r="G54" s="15"/>
-      <c r="H54" s="15"/>
-      <c r="I54" s="15"/>
-      <c r="J54" s="15"/>
+      <c r="A54" s="16"/>
+      <c r="B54" s="16"/>
+      <c r="C54" s="16"/>
+      <c r="D54" s="16"/>
+      <c r="E54" s="16"/>
+      <c r="F54" s="16"/>
+      <c r="G54" s="16"/>
+      <c r="H54" s="16"/>
+      <c r="I54" s="16"/>
+      <c r="J54" s="16"/>
       <c r="K54" s="3" t="s">
         <v>192</v>
       </c>
@@ -6975,16 +6987,16 @@
       <c r="AA54" s="2"/>
     </row>
     <row r="55" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="15"/>
-      <c r="B55" s="15"/>
-      <c r="C55" s="15"/>
-      <c r="D55" s="15"/>
-      <c r="E55" s="15"/>
-      <c r="F55" s="15"/>
-      <c r="G55" s="15"/>
-      <c r="H55" s="15"/>
-      <c r="I55" s="15"/>
-      <c r="J55" s="15"/>
+      <c r="A55" s="16"/>
+      <c r="B55" s="16"/>
+      <c r="C55" s="16"/>
+      <c r="D55" s="16"/>
+      <c r="E55" s="16"/>
+      <c r="F55" s="16"/>
+      <c r="G55" s="16"/>
+      <c r="H55" s="16"/>
+      <c r="I55" s="16"/>
+      <c r="J55" s="16"/>
       <c r="K55" s="3" t="s">
         <v>193</v>
       </c>
@@ -7006,16 +7018,16 @@
       <c r="AA55" s="2"/>
     </row>
     <row r="56" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="15"/>
-      <c r="B56" s="15"/>
-      <c r="C56" s="15"/>
-      <c r="D56" s="15"/>
-      <c r="E56" s="15"/>
-      <c r="F56" s="15"/>
-      <c r="G56" s="15"/>
-      <c r="H56" s="15"/>
-      <c r="I56" s="15"/>
-      <c r="J56" s="15"/>
+      <c r="A56" s="16"/>
+      <c r="B56" s="16"/>
+      <c r="C56" s="16"/>
+      <c r="D56" s="16"/>
+      <c r="E56" s="16"/>
+      <c r="F56" s="16"/>
+      <c r="G56" s="16"/>
+      <c r="H56" s="16"/>
+      <c r="I56" s="16"/>
+      <c r="J56" s="16"/>
       <c r="K56" s="3" t="s">
         <v>194</v>
       </c>
@@ -7037,16 +7049,16 @@
       <c r="AA56" s="2"/>
     </row>
     <row r="57" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="15"/>
-      <c r="B57" s="15"/>
-      <c r="C57" s="15"/>
-      <c r="D57" s="15"/>
-      <c r="E57" s="15"/>
-      <c r="F57" s="15"/>
-      <c r="G57" s="15"/>
-      <c r="H57" s="15"/>
-      <c r="I57" s="15"/>
-      <c r="J57" s="15"/>
+      <c r="A57" s="16"/>
+      <c r="B57" s="16"/>
+      <c r="C57" s="16"/>
+      <c r="D57" s="16"/>
+      <c r="E57" s="16"/>
+      <c r="F57" s="16"/>
+      <c r="G57" s="16"/>
+      <c r="H57" s="16"/>
+      <c r="I57" s="16"/>
+      <c r="J57" s="16"/>
       <c r="K57" s="3" t="s">
         <v>195</v>
       </c>
@@ -7068,16 +7080,16 @@
       <c r="AA57" s="2"/>
     </row>
     <row r="58" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="15"/>
-      <c r="B58" s="15"/>
-      <c r="C58" s="15"/>
-      <c r="D58" s="15"/>
-      <c r="E58" s="15"/>
-      <c r="F58" s="15"/>
-      <c r="G58" s="15"/>
-      <c r="H58" s="15"/>
-      <c r="I58" s="15"/>
-      <c r="J58" s="15"/>
+      <c r="A58" s="16"/>
+      <c r="B58" s="16"/>
+      <c r="C58" s="16"/>
+      <c r="D58" s="16"/>
+      <c r="E58" s="16"/>
+      <c r="F58" s="16"/>
+      <c r="G58" s="16"/>
+      <c r="H58" s="16"/>
+      <c r="I58" s="16"/>
+      <c r="J58" s="16"/>
       <c r="K58" s="3" t="s">
         <v>196</v>
       </c>
@@ -7099,16 +7111,16 @@
       <c r="AA58" s="2"/>
     </row>
     <row r="59" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="15"/>
-      <c r="B59" s="15"/>
-      <c r="C59" s="15"/>
-      <c r="D59" s="15"/>
-      <c r="E59" s="15"/>
-      <c r="F59" s="15"/>
-      <c r="G59" s="15"/>
-      <c r="H59" s="15"/>
-      <c r="I59" s="15"/>
-      <c r="J59" s="15"/>
+      <c r="A59" s="16"/>
+      <c r="B59" s="16"/>
+      <c r="C59" s="16"/>
+      <c r="D59" s="16"/>
+      <c r="E59" s="16"/>
+      <c r="F59" s="16"/>
+      <c r="G59" s="16"/>
+      <c r="H59" s="16"/>
+      <c r="I59" s="16"/>
+      <c r="J59" s="16"/>
       <c r="K59" s="3" t="s">
         <v>197</v>
       </c>
@@ -7130,16 +7142,16 @@
       <c r="AA59" s="2"/>
     </row>
     <row r="60" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="15"/>
-      <c r="B60" s="15"/>
-      <c r="C60" s="15"/>
-      <c r="D60" s="15"/>
-      <c r="E60" s="15"/>
-      <c r="F60" s="15"/>
-      <c r="G60" s="15"/>
-      <c r="H60" s="15"/>
-      <c r="I60" s="15"/>
-      <c r="J60" s="15"/>
+      <c r="A60" s="16"/>
+      <c r="B60" s="16"/>
+      <c r="C60" s="16"/>
+      <c r="D60" s="16"/>
+      <c r="E60" s="16"/>
+      <c r="F60" s="16"/>
+      <c r="G60" s="16"/>
+      <c r="H60" s="16"/>
+      <c r="I60" s="16"/>
+      <c r="J60" s="16"/>
       <c r="K60" s="3" t="s">
         <v>198</v>
       </c>
@@ -7161,16 +7173,16 @@
       <c r="AA60" s="2"/>
     </row>
     <row r="61" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="15"/>
-      <c r="B61" s="15"/>
-      <c r="C61" s="15"/>
-      <c r="D61" s="15"/>
-      <c r="E61" s="15"/>
-      <c r="F61" s="15"/>
-      <c r="G61" s="15"/>
-      <c r="H61" s="15"/>
-      <c r="I61" s="15"/>
-      <c r="J61" s="15"/>
+      <c r="A61" s="16"/>
+      <c r="B61" s="16"/>
+      <c r="C61" s="16"/>
+      <c r="D61" s="16"/>
+      <c r="E61" s="16"/>
+      <c r="F61" s="16"/>
+      <c r="G61" s="16"/>
+      <c r="H61" s="16"/>
+      <c r="I61" s="16"/>
+      <c r="J61" s="16"/>
       <c r="K61" s="3" t="s">
         <v>199</v>
       </c>
@@ -7192,16 +7204,16 @@
       <c r="AA61" s="2"/>
     </row>
     <row r="62" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="15"/>
-      <c r="B62" s="15"/>
-      <c r="C62" s="15"/>
-      <c r="D62" s="15"/>
-      <c r="E62" s="15"/>
-      <c r="F62" s="15"/>
-      <c r="G62" s="15"/>
-      <c r="H62" s="15"/>
-      <c r="I62" s="15"/>
-      <c r="J62" s="15"/>
+      <c r="A62" s="16"/>
+      <c r="B62" s="16"/>
+      <c r="C62" s="16"/>
+      <c r="D62" s="16"/>
+      <c r="E62" s="16"/>
+      <c r="F62" s="16"/>
+      <c r="G62" s="16"/>
+      <c r="H62" s="16"/>
+      <c r="I62" s="16"/>
+      <c r="J62" s="16"/>
       <c r="K62" s="3" t="s">
         <v>200</v>
       </c>
@@ -7223,16 +7235,16 @@
       <c r="AA62" s="2"/>
     </row>
     <row r="63" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="15"/>
-      <c r="B63" s="15"/>
-      <c r="C63" s="15"/>
-      <c r="D63" s="15"/>
-      <c r="E63" s="15"/>
-      <c r="F63" s="15"/>
-      <c r="G63" s="15"/>
-      <c r="H63" s="15"/>
-      <c r="I63" s="15"/>
-      <c r="J63" s="15"/>
+      <c r="A63" s="16"/>
+      <c r="B63" s="16"/>
+      <c r="C63" s="16"/>
+      <c r="D63" s="16"/>
+      <c r="E63" s="16"/>
+      <c r="F63" s="16"/>
+      <c r="G63" s="16"/>
+      <c r="H63" s="16"/>
+      <c r="I63" s="16"/>
+      <c r="J63" s="16"/>
       <c r="K63" s="3" t="s">
         <v>201</v>
       </c>
@@ -7254,16 +7266,16 @@
       <c r="AA63" s="2"/>
     </row>
     <row r="64" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="15"/>
-      <c r="B64" s="15"/>
-      <c r="C64" s="15"/>
-      <c r="D64" s="15"/>
-      <c r="E64" s="15"/>
-      <c r="F64" s="15"/>
-      <c r="G64" s="15"/>
-      <c r="H64" s="15"/>
-      <c r="I64" s="15"/>
-      <c r="J64" s="15"/>
+      <c r="A64" s="16"/>
+      <c r="B64" s="16"/>
+      <c r="C64" s="16"/>
+      <c r="D64" s="16"/>
+      <c r="E64" s="16"/>
+      <c r="F64" s="16"/>
+      <c r="G64" s="16"/>
+      <c r="H64" s="16"/>
+      <c r="I64" s="16"/>
+      <c r="J64" s="16"/>
       <c r="K64" s="3" t="s">
         <v>202</v>
       </c>
@@ -7285,16 +7297,16 @@
       <c r="AA64" s="2"/>
     </row>
     <row r="65" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="15"/>
-      <c r="B65" s="15"/>
-      <c r="C65" s="15"/>
-      <c r="D65" s="15"/>
-      <c r="E65" s="15"/>
-      <c r="F65" s="15"/>
-      <c r="G65" s="15"/>
-      <c r="H65" s="15"/>
-      <c r="I65" s="15"/>
-      <c r="J65" s="15"/>
+      <c r="A65" s="16"/>
+      <c r="B65" s="16"/>
+      <c r="C65" s="16"/>
+      <c r="D65" s="16"/>
+      <c r="E65" s="16"/>
+      <c r="F65" s="16"/>
+      <c r="G65" s="16"/>
+      <c r="H65" s="16"/>
+      <c r="I65" s="16"/>
+      <c r="J65" s="16"/>
       <c r="K65" s="3" t="s">
         <v>203</v>
       </c>
@@ -7316,16 +7328,16 @@
       <c r="AA65" s="2"/>
     </row>
     <row r="66" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="15"/>
-      <c r="B66" s="15"/>
-      <c r="C66" s="15"/>
-      <c r="D66" s="15"/>
-      <c r="E66" s="15"/>
-      <c r="F66" s="15"/>
-      <c r="G66" s="15"/>
-      <c r="H66" s="15"/>
-      <c r="I66" s="15"/>
-      <c r="J66" s="15"/>
+      <c r="A66" s="16"/>
+      <c r="B66" s="16"/>
+      <c r="C66" s="16"/>
+      <c r="D66" s="16"/>
+      <c r="E66" s="16"/>
+      <c r="F66" s="16"/>
+      <c r="G66" s="16"/>
+      <c r="H66" s="16"/>
+      <c r="I66" s="16"/>
+      <c r="J66" s="16"/>
       <c r="K66" s="3" t="s">
         <v>204</v>
       </c>
@@ -7347,16 +7359,16 @@
       <c r="AA66" s="2"/>
     </row>
     <row r="67" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="15"/>
-      <c r="B67" s="15"/>
-      <c r="C67" s="15"/>
-      <c r="D67" s="15"/>
-      <c r="E67" s="15"/>
-      <c r="F67" s="15"/>
-      <c r="G67" s="15"/>
-      <c r="H67" s="15"/>
-      <c r="I67" s="15"/>
-      <c r="J67" s="15"/>
+      <c r="A67" s="16"/>
+      <c r="B67" s="16"/>
+      <c r="C67" s="16"/>
+      <c r="D67" s="16"/>
+      <c r="E67" s="16"/>
+      <c r="F67" s="16"/>
+      <c r="G67" s="16"/>
+      <c r="H67" s="16"/>
+      <c r="I67" s="16"/>
+      <c r="J67" s="16"/>
       <c r="K67" s="3" t="s">
         <v>205</v>
       </c>
@@ -7378,16 +7390,16 @@
       <c r="AA67" s="2"/>
     </row>
     <row r="68" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="15"/>
-      <c r="B68" s="15"/>
-      <c r="C68" s="15"/>
-      <c r="D68" s="15"/>
-      <c r="E68" s="15"/>
-      <c r="F68" s="15"/>
-      <c r="G68" s="15"/>
-      <c r="H68" s="15"/>
-      <c r="I68" s="15"/>
-      <c r="J68" s="15"/>
+      <c r="A68" s="16"/>
+      <c r="B68" s="16"/>
+      <c r="C68" s="16"/>
+      <c r="D68" s="16"/>
+      <c r="E68" s="16"/>
+      <c r="F68" s="16"/>
+      <c r="G68" s="16"/>
+      <c r="H68" s="16"/>
+      <c r="I68" s="16"/>
+      <c r="J68" s="16"/>
       <c r="K68" s="3" t="s">
         <v>206</v>
       </c>
@@ -7409,16 +7421,16 @@
       <c r="AA68" s="2"/>
     </row>
     <row r="69" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="15"/>
-      <c r="B69" s="15"/>
-      <c r="C69" s="15"/>
-      <c r="D69" s="15"/>
-      <c r="E69" s="15"/>
-      <c r="F69" s="15"/>
-      <c r="G69" s="15"/>
-      <c r="H69" s="15"/>
-      <c r="I69" s="15"/>
-      <c r="J69" s="15"/>
+      <c r="A69" s="16"/>
+      <c r="B69" s="16"/>
+      <c r="C69" s="16"/>
+      <c r="D69" s="16"/>
+      <c r="E69" s="16"/>
+      <c r="F69" s="16"/>
+      <c r="G69" s="16"/>
+      <c r="H69" s="16"/>
+      <c r="I69" s="16"/>
+      <c r="J69" s="16"/>
       <c r="K69" s="3" t="s">
         <v>207</v>
       </c>
@@ -7440,16 +7452,16 @@
       <c r="AA69" s="2"/>
     </row>
     <row r="70" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="15"/>
-      <c r="B70" s="15"/>
-      <c r="C70" s="15"/>
-      <c r="D70" s="15"/>
-      <c r="E70" s="15"/>
-      <c r="F70" s="15"/>
-      <c r="G70" s="15"/>
-      <c r="H70" s="15"/>
-      <c r="I70" s="15"/>
-      <c r="J70" s="15"/>
+      <c r="A70" s="16"/>
+      <c r="B70" s="16"/>
+      <c r="C70" s="16"/>
+      <c r="D70" s="16"/>
+      <c r="E70" s="16"/>
+      <c r="F70" s="16"/>
+      <c r="G70" s="16"/>
+      <c r="H70" s="16"/>
+      <c r="I70" s="16"/>
+      <c r="J70" s="16"/>
       <c r="K70" s="3"/>
       <c r="L70" s="2"/>
       <c r="M70" s="2"/>
@@ -7469,16 +7481,16 @@
       <c r="AA70" s="2"/>
     </row>
     <row r="71" spans="1:27" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="13"/>
-      <c r="B71" s="13"/>
-      <c r="C71" s="13"/>
-      <c r="D71" s="13"/>
-      <c r="E71" s="13"/>
-      <c r="F71" s="13"/>
-      <c r="G71" s="13"/>
-      <c r="H71" s="13"/>
-      <c r="I71" s="13"/>
-      <c r="J71" s="13"/>
+      <c r="A71" s="17"/>
+      <c r="B71" s="17"/>
+      <c r="C71" s="17"/>
+      <c r="D71" s="17"/>
+      <c r="E71" s="17"/>
+      <c r="F71" s="17"/>
+      <c r="G71" s="17"/>
+      <c r="H71" s="17"/>
+      <c r="I71" s="17"/>
+      <c r="J71" s="17"/>
       <c r="K71" s="4" t="s">
         <v>208</v>
       </c>
@@ -7499,31 +7511,31 @@
       <c r="Z71" s="2"/>
       <c r="AA71" s="2"/>
     </row>
-    <row r="72" spans="1:27" s="24" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="22"/>
-      <c r="B72" s="23" t="s">
+    <row r="72" spans="1:27" s="14" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A72" s="12"/>
+      <c r="B72" s="13" t="s">
         <v>520</v>
       </c>
-      <c r="C72" s="23" t="s">
+      <c r="C72" s="13" t="s">
         <v>519</v>
       </c>
-      <c r="D72" s="23">
+      <c r="D72" s="13">
         <v>14</v>
       </c>
-      <c r="E72" s="23">
+      <c r="E72" s="13">
         <v>2629</v>
       </c>
-      <c r="F72" s="23" t="s">
+      <c r="F72" s="13" t="s">
         <v>518</v>
       </c>
-      <c r="G72" s="23" t="s">
+      <c r="G72" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="H72" s="23" t="s">
+      <c r="H72" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="I72" s="23"/>
-      <c r="J72" s="23"/>
+      <c r="I72" s="13"/>
+      <c r="J72" s="13"/>
       <c r="K72" s="4" t="s">
         <v>521</v>
       </c>
@@ -7680,32 +7692,32 @@
       <c r="AA75" s="2"/>
     </row>
     <row r="76" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="14" t="s">
+      <c r="A76" s="18" t="s">
         <v>219</v>
       </c>
-      <c r="B76" s="12" t="s">
+      <c r="B76" s="15" t="s">
         <v>220</v>
       </c>
       <c r="C76" s="19" t="s">
         <v>221</v>
       </c>
-      <c r="D76" s="12">
+      <c r="D76" s="15">
         <v>10</v>
       </c>
-      <c r="E76" s="12">
+      <c r="E76" s="15">
         <v>1153</v>
       </c>
-      <c r="F76" s="12" t="s">
+      <c r="F76" s="15" t="s">
         <v>222</v>
       </c>
-      <c r="G76" s="12" t="s">
+      <c r="G76" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="H76" s="12" t="s">
+      <c r="H76" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="I76" s="12"/>
-      <c r="J76" s="12"/>
+      <c r="I76" s="15"/>
+      <c r="J76" s="15"/>
       <c r="K76" s="3" t="s">
         <v>223</v>
       </c>
@@ -7727,16 +7739,16 @@
       <c r="AA76" s="2"/>
     </row>
     <row r="77" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="15"/>
-      <c r="B77" s="15"/>
-      <c r="C77" s="15"/>
-      <c r="D77" s="15"/>
-      <c r="E77" s="15"/>
-      <c r="F77" s="15"/>
-      <c r="G77" s="15"/>
-      <c r="H77" s="15"/>
-      <c r="I77" s="15"/>
-      <c r="J77" s="15"/>
+      <c r="A77" s="16"/>
+      <c r="B77" s="16"/>
+      <c r="C77" s="16"/>
+      <c r="D77" s="16"/>
+      <c r="E77" s="16"/>
+      <c r="F77" s="16"/>
+      <c r="G77" s="16"/>
+      <c r="H77" s="16"/>
+      <c r="I77" s="16"/>
+      <c r="J77" s="16"/>
       <c r="K77" s="3" t="s">
         <v>224</v>
       </c>
@@ -7758,16 +7770,16 @@
       <c r="AA77" s="2"/>
     </row>
     <row r="78" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="15"/>
-      <c r="B78" s="15"/>
-      <c r="C78" s="15"/>
-      <c r="D78" s="15"/>
-      <c r="E78" s="15"/>
-      <c r="F78" s="15"/>
-      <c r="G78" s="15"/>
-      <c r="H78" s="15"/>
-      <c r="I78" s="15"/>
-      <c r="J78" s="15"/>
+      <c r="A78" s="16"/>
+      <c r="B78" s="16"/>
+      <c r="C78" s="16"/>
+      <c r="D78" s="16"/>
+      <c r="E78" s="16"/>
+      <c r="F78" s="16"/>
+      <c r="G78" s="16"/>
+      <c r="H78" s="16"/>
+      <c r="I78" s="16"/>
+      <c r="J78" s="16"/>
       <c r="K78" s="3" t="s">
         <v>225</v>
       </c>
@@ -7789,16 +7801,16 @@
       <c r="AA78" s="2"/>
     </row>
     <row r="79" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="15"/>
-      <c r="B79" s="15"/>
-      <c r="C79" s="15"/>
-      <c r="D79" s="15"/>
-      <c r="E79" s="15"/>
-      <c r="F79" s="15"/>
-      <c r="G79" s="15"/>
-      <c r="H79" s="15"/>
-      <c r="I79" s="15"/>
-      <c r="J79" s="15"/>
+      <c r="A79" s="16"/>
+      <c r="B79" s="16"/>
+      <c r="C79" s="16"/>
+      <c r="D79" s="16"/>
+      <c r="E79" s="16"/>
+      <c r="F79" s="16"/>
+      <c r="G79" s="16"/>
+      <c r="H79" s="16"/>
+      <c r="I79" s="16"/>
+      <c r="J79" s="16"/>
       <c r="L79" s="2"/>
       <c r="M79" s="2"/>
       <c r="N79" s="2"/>
@@ -7817,16 +7829,16 @@
       <c r="AA79" s="2"/>
     </row>
     <row r="80" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="13"/>
-      <c r="B80" s="13"/>
-      <c r="C80" s="13"/>
-      <c r="D80" s="13"/>
-      <c r="E80" s="13"/>
-      <c r="F80" s="13"/>
-      <c r="G80" s="13"/>
-      <c r="H80" s="13"/>
-      <c r="I80" s="13"/>
-      <c r="J80" s="13"/>
+      <c r="A80" s="17"/>
+      <c r="B80" s="17"/>
+      <c r="C80" s="17"/>
+      <c r="D80" s="17"/>
+      <c r="E80" s="17"/>
+      <c r="F80" s="17"/>
+      <c r="G80" s="17"/>
+      <c r="H80" s="17"/>
+      <c r="I80" s="17"/>
+      <c r="J80" s="17"/>
       <c r="K80" s="4" t="s">
         <v>226</v>
       </c>
@@ -7848,30 +7860,30 @@
       <c r="AA80" s="2"/>
     </row>
     <row r="81" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="14" t="s">
+      <c r="A81" s="18" t="s">
         <v>227</v>
       </c>
-      <c r="B81" s="12" t="s">
+      <c r="B81" s="15" t="s">
         <v>228</v>
       </c>
       <c r="C81" s="19" t="s">
         <v>229</v>
       </c>
-      <c r="D81" s="12">
+      <c r="D81" s="15">
         <v>44</v>
       </c>
-      <c r="E81" s="12">
+      <c r="E81" s="15">
         <v>3709</v>
       </c>
-      <c r="F81" s="12" t="s">
+      <c r="F81" s="15" t="s">
         <v>230</v>
       </c>
-      <c r="G81" s="12" t="s">
+      <c r="G81" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="H81" s="12"/>
-      <c r="I81" s="12"/>
-      <c r="J81" s="12"/>
+      <c r="H81" s="15"/>
+      <c r="I81" s="15"/>
+      <c r="J81" s="15"/>
       <c r="K81" s="3" t="s">
         <v>231</v>
       </c>
@@ -7893,16 +7905,16 @@
       <c r="AA81" s="2"/>
     </row>
     <row r="82" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="15"/>
-      <c r="B82" s="15"/>
-      <c r="C82" s="15"/>
-      <c r="D82" s="15"/>
-      <c r="E82" s="15"/>
-      <c r="F82" s="15"/>
-      <c r="G82" s="15"/>
-      <c r="H82" s="15"/>
-      <c r="I82" s="15"/>
-      <c r="J82" s="15"/>
+      <c r="A82" s="16"/>
+      <c r="B82" s="16"/>
+      <c r="C82" s="16"/>
+      <c r="D82" s="16"/>
+      <c r="E82" s="16"/>
+      <c r="F82" s="16"/>
+      <c r="G82" s="16"/>
+      <c r="H82" s="16"/>
+      <c r="I82" s="16"/>
+      <c r="J82" s="16"/>
       <c r="K82" s="3" t="s">
         <v>232</v>
       </c>
@@ -7924,16 +7936,16 @@
       <c r="AA82" s="2"/>
     </row>
     <row r="83" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="15"/>
-      <c r="B83" s="15"/>
-      <c r="C83" s="15"/>
-      <c r="D83" s="15"/>
-      <c r="E83" s="15"/>
-      <c r="F83" s="15"/>
-      <c r="G83" s="15"/>
-      <c r="H83" s="15"/>
-      <c r="I83" s="15"/>
-      <c r="J83" s="15"/>
+      <c r="A83" s="16"/>
+      <c r="B83" s="16"/>
+      <c r="C83" s="16"/>
+      <c r="D83" s="16"/>
+      <c r="E83" s="16"/>
+      <c r="F83" s="16"/>
+      <c r="G83" s="16"/>
+      <c r="H83" s="16"/>
+      <c r="I83" s="16"/>
+      <c r="J83" s="16"/>
       <c r="K83" s="3" t="s">
         <v>233</v>
       </c>
@@ -7955,16 +7967,16 @@
       <c r="AA83" s="2"/>
     </row>
     <row r="84" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="13"/>
-      <c r="B84" s="13"/>
-      <c r="C84" s="13"/>
-      <c r="D84" s="13"/>
-      <c r="E84" s="13"/>
-      <c r="F84" s="13"/>
-      <c r="G84" s="13"/>
-      <c r="H84" s="13"/>
-      <c r="I84" s="13"/>
-      <c r="J84" s="13"/>
+      <c r="A84" s="17"/>
+      <c r="B84" s="17"/>
+      <c r="C84" s="17"/>
+      <c r="D84" s="17"/>
+      <c r="E84" s="17"/>
+      <c r="F84" s="17"/>
+      <c r="G84" s="17"/>
+      <c r="H84" s="17"/>
+      <c r="I84" s="17"/>
+      <c r="J84" s="17"/>
       <c r="K84" s="4" t="s">
         <v>234</v>
       </c>
@@ -7986,13 +7998,13 @@
       <c r="AA84" s="2"/>
     </row>
     <row r="85" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="14" t="s">
+      <c r="A85" s="18" t="s">
         <v>235</v>
       </c>
-      <c r="B85" s="12" t="s">
+      <c r="B85" s="15" t="s">
         <v>236</v>
       </c>
-      <c r="C85" s="16" t="s">
+      <c r="C85" s="22" t="s">
         <v>237</v>
       </c>
       <c r="D85" s="4">
@@ -8033,9 +8045,9 @@
       <c r="AA85" s="2"/>
     </row>
     <row r="86" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="15"/>
-      <c r="B86" s="15"/>
-      <c r="C86" s="17"/>
+      <c r="A86" s="16"/>
+      <c r="B86" s="16"/>
+      <c r="C86" s="23"/>
       <c r="D86" s="4">
         <v>263</v>
       </c>
@@ -8074,9 +8086,9 @@
       <c r="AA86" s="2"/>
     </row>
     <row r="87" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A87" s="15"/>
-      <c r="B87" s="15"/>
-      <c r="C87" s="17"/>
+      <c r="A87" s="16"/>
+      <c r="B87" s="16"/>
+      <c r="C87" s="23"/>
       <c r="D87" s="4">
         <v>144</v>
       </c>
@@ -8115,9 +8127,9 @@
       <c r="AA87" s="2"/>
     </row>
     <row r="88" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A88" s="13"/>
-      <c r="B88" s="13"/>
-      <c r="C88" s="18"/>
+      <c r="A88" s="17"/>
+      <c r="B88" s="17"/>
+      <c r="C88" s="24"/>
       <c r="D88" s="4">
         <v>254</v>
       </c>
@@ -9282,24 +9294,24 @@
       <c r="AA118" s="2"/>
     </row>
     <row r="119" spans="1:27" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A119" s="14" t="s">
+      <c r="A119" s="18" t="s">
         <v>371</v>
       </c>
-      <c r="B119" s="12" t="s">
+      <c r="B119" s="15" t="s">
         <v>372</v>
       </c>
       <c r="C119" s="19" t="s">
         <v>373</v>
       </c>
-      <c r="D119" s="12"/>
-      <c r="E119" s="12"/>
-      <c r="F119" s="12" t="s">
+      <c r="D119" s="15"/>
+      <c r="E119" s="15"/>
+      <c r="F119" s="15" t="s">
         <v>374</v>
       </c>
-      <c r="G119" s="12"/>
-      <c r="H119" s="12"/>
-      <c r="I119" s="12"/>
-      <c r="J119" s="12"/>
+      <c r="G119" s="15"/>
+      <c r="H119" s="15"/>
+      <c r="I119" s="15"/>
+      <c r="J119" s="15"/>
       <c r="K119" s="3" t="s">
         <v>375</v>
       </c>
@@ -9321,16 +9333,16 @@
       <c r="AA119" s="2"/>
     </row>
     <row r="120" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A120" s="13"/>
-      <c r="B120" s="13"/>
-      <c r="C120" s="13"/>
-      <c r="D120" s="13"/>
-      <c r="E120" s="13"/>
-      <c r="F120" s="13"/>
-      <c r="G120" s="13"/>
-      <c r="H120" s="13"/>
-      <c r="I120" s="13"/>
-      <c r="J120" s="13"/>
+      <c r="A120" s="17"/>
+      <c r="B120" s="17"/>
+      <c r="C120" s="17"/>
+      <c r="D120" s="17"/>
+      <c r="E120" s="17"/>
+      <c r="F120" s="17"/>
+      <c r="G120" s="17"/>
+      <c r="H120" s="17"/>
+      <c r="I120" s="17"/>
+      <c r="J120" s="17"/>
       <c r="K120" s="4" t="s">
         <v>376</v>
       </c>
@@ -9538,7 +9550,7 @@
       <c r="Z125" s="2"/>
       <c r="AA125" s="2"/>
     </row>
-    <row r="126" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:27" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A126" s="5" t="s">
         <v>398</v>
       </c>
@@ -9577,26 +9589,26 @@
       <c r="Z126" s="2"/>
       <c r="AA126" s="2"/>
     </row>
-    <row r="127" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A127" s="5" t="s">
-        <v>403</v>
-      </c>
+    <row r="127" spans="1:27" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A127" s="5"/>
       <c r="B127" s="4" t="s">
-        <v>404</v>
+        <v>522</v>
       </c>
       <c r="C127" s="6" t="s">
-        <v>405</v>
+        <v>524</v>
       </c>
       <c r="D127" s="4"/>
       <c r="E127" s="4"/>
       <c r="F127" s="4" t="s">
-        <v>406</v>
+        <v>523</v>
       </c>
       <c r="G127" s="4"/>
       <c r="H127" s="4"/>
       <c r="I127" s="4"/>
       <c r="J127" s="4"/>
-      <c r="K127" s="4"/>
+      <c r="K127" s="4" t="s">
+        <v>525</v>
+      </c>
       <c r="L127" s="2"/>
       <c r="M127" s="2"/>
       <c r="N127" s="2"/>
@@ -9614,20 +9626,20 @@
       <c r="Z127" s="2"/>
       <c r="AA127" s="2"/>
     </row>
-    <row r="128" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:27" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A128" s="5" t="s">
-        <v>407</v>
+        <v>403</v>
       </c>
       <c r="B128" s="4" t="s">
-        <v>408</v>
+        <v>404</v>
       </c>
       <c r="C128" s="6" t="s">
-        <v>409</v>
+        <v>405</v>
       </c>
       <c r="D128" s="4"/>
       <c r="E128" s="4"/>
       <c r="F128" s="4" t="s">
-        <v>410</v>
+        <v>406</v>
       </c>
       <c r="G128" s="4"/>
       <c r="H128" s="4"/>
@@ -9653,18 +9665,18 @@
     </row>
     <row r="129" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A129" s="5" t="s">
-        <v>411</v>
+        <v>407</v>
       </c>
       <c r="B129" s="4" t="s">
-        <v>412</v>
+        <v>408</v>
       </c>
       <c r="C129" s="6" t="s">
-        <v>413</v>
+        <v>409</v>
       </c>
       <c r="D129" s="4"/>
       <c r="E129" s="4"/>
       <c r="F129" s="4" t="s">
-        <v>414</v>
+        <v>410</v>
       </c>
       <c r="G129" s="4"/>
       <c r="H129" s="4"/>
@@ -9690,18 +9702,18 @@
     </row>
     <row r="130" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A130" s="5" t="s">
-        <v>415</v>
+        <v>411</v>
       </c>
       <c r="B130" s="4" t="s">
-        <v>416</v>
+        <v>412</v>
       </c>
       <c r="C130" s="6" t="s">
-        <v>417</v>
+        <v>413</v>
       </c>
       <c r="D130" s="4"/>
       <c r="E130" s="4"/>
       <c r="F130" s="4" t="s">
-        <v>418</v>
+        <v>414</v>
       </c>
       <c r="G130" s="4"/>
       <c r="H130" s="4"/>
@@ -9727,18 +9739,18 @@
     </row>
     <row r="131" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A131" s="5" t="s">
-        <v>419</v>
+        <v>415</v>
       </c>
       <c r="B131" s="4" t="s">
-        <v>420</v>
+        <v>416</v>
       </c>
       <c r="C131" s="6" t="s">
-        <v>421</v>
+        <v>417</v>
       </c>
       <c r="D131" s="4"/>
       <c r="E131" s="4"/>
       <c r="F131" s="4" t="s">
-        <v>422</v>
+        <v>418</v>
       </c>
       <c r="G131" s="4"/>
       <c r="H131" s="4"/>
@@ -9764,18 +9776,18 @@
     </row>
     <row r="132" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A132" s="5" t="s">
-        <v>423</v>
+        <v>419</v>
       </c>
       <c r="B132" s="4" t="s">
-        <v>424</v>
+        <v>420</v>
       </c>
       <c r="C132" s="6" t="s">
-        <v>425</v>
+        <v>421</v>
       </c>
       <c r="D132" s="4"/>
       <c r="E132" s="4"/>
       <c r="F132" s="4" t="s">
-        <v>426</v>
+        <v>422</v>
       </c>
       <c r="G132" s="4"/>
       <c r="H132" s="4"/>
@@ -9801,18 +9813,18 @@
     </row>
     <row r="133" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A133" s="5" t="s">
-        <v>427</v>
+        <v>423</v>
       </c>
       <c r="B133" s="4" t="s">
-        <v>428</v>
+        <v>424</v>
       </c>
       <c r="C133" s="6" t="s">
-        <v>429</v>
+        <v>425</v>
       </c>
       <c r="D133" s="4"/>
       <c r="E133" s="4"/>
       <c r="F133" s="4" t="s">
-        <v>430</v>
+        <v>426</v>
       </c>
       <c r="G133" s="4"/>
       <c r="H133" s="4"/>
@@ -9838,18 +9850,18 @@
     </row>
     <row r="134" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A134" s="5" t="s">
-        <v>431</v>
+        <v>427</v>
       </c>
       <c r="B134" s="4" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
       <c r="C134" s="6" t="s">
-        <v>433</v>
+        <v>429</v>
       </c>
       <c r="D134" s="4"/>
       <c r="E134" s="4"/>
       <c r="F134" s="4" t="s">
-        <v>434</v>
+        <v>430</v>
       </c>
       <c r="G134" s="4"/>
       <c r="H134" s="4"/>
@@ -9875,18 +9887,18 @@
     </row>
     <row r="135" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A135" s="5" t="s">
-        <v>435</v>
+        <v>431</v>
       </c>
       <c r="B135" s="4" t="s">
-        <v>436</v>
+        <v>432</v>
       </c>
       <c r="C135" s="6" t="s">
-        <v>437</v>
+        <v>433</v>
       </c>
       <c r="D135" s="4"/>
       <c r="E135" s="4"/>
       <c r="F135" s="4" t="s">
-        <v>438</v>
+        <v>434</v>
       </c>
       <c r="G135" s="4"/>
       <c r="H135" s="4"/>
@@ -9912,18 +9924,18 @@
     </row>
     <row r="136" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A136" s="5" t="s">
-        <v>439</v>
+        <v>435</v>
       </c>
       <c r="B136" s="4" t="s">
-        <v>440</v>
+        <v>436</v>
       </c>
       <c r="C136" s="6" t="s">
-        <v>441</v>
+        <v>437</v>
       </c>
       <c r="D136" s="4"/>
       <c r="E136" s="4"/>
       <c r="F136" s="4" t="s">
-        <v>442</v>
+        <v>438</v>
       </c>
       <c r="G136" s="4"/>
       <c r="H136" s="4"/>
@@ -9949,18 +9961,18 @@
     </row>
     <row r="137" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A137" s="5" t="s">
-        <v>443</v>
+        <v>439</v>
       </c>
       <c r="B137" s="4" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="C137" s="6" t="s">
-        <v>445</v>
+        <v>441</v>
       </c>
       <c r="D137" s="4"/>
       <c r="E137" s="4"/>
       <c r="F137" s="4" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="G137" s="4"/>
       <c r="H137" s="4"/>
@@ -9986,18 +9998,18 @@
     </row>
     <row r="138" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A138" s="5" t="s">
-        <v>447</v>
+        <v>443</v>
       </c>
       <c r="B138" s="4" t="s">
-        <v>448</v>
+        <v>444</v>
       </c>
       <c r="C138" s="6" t="s">
-        <v>449</v>
+        <v>445</v>
       </c>
       <c r="D138" s="4"/>
       <c r="E138" s="4"/>
       <c r="F138" s="4" t="s">
-        <v>450</v>
+        <v>446</v>
       </c>
       <c r="G138" s="4"/>
       <c r="H138" s="4"/>
@@ -10023,18 +10035,18 @@
     </row>
     <row r="139" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A139" s="5" t="s">
-        <v>451</v>
+        <v>447</v>
       </c>
       <c r="B139" s="4" t="s">
-        <v>452</v>
+        <v>448</v>
       </c>
       <c r="C139" s="6" t="s">
-        <v>453</v>
+        <v>449</v>
       </c>
       <c r="D139" s="4"/>
       <c r="E139" s="4"/>
       <c r="F139" s="4" t="s">
-        <v>454</v>
+        <v>450</v>
       </c>
       <c r="G139" s="4"/>
       <c r="H139" s="4"/>
@@ -10060,18 +10072,18 @@
     </row>
     <row r="140" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A140" s="5" t="s">
-        <v>455</v>
+        <v>451</v>
       </c>
       <c r="B140" s="4" t="s">
-        <v>456</v>
+        <v>452</v>
       </c>
       <c r="C140" s="6" t="s">
-        <v>457</v>
+        <v>453</v>
       </c>
       <c r="D140" s="4"/>
       <c r="E140" s="4"/>
       <c r="F140" s="4" t="s">
-        <v>458</v>
+        <v>454</v>
       </c>
       <c r="G140" s="4"/>
       <c r="H140" s="4"/>
@@ -10097,18 +10109,18 @@
     </row>
     <row r="141" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A141" s="5" t="s">
-        <v>459</v>
+        <v>455</v>
       </c>
       <c r="B141" s="4" t="s">
-        <v>460</v>
+        <v>456</v>
       </c>
       <c r="C141" s="6" t="s">
-        <v>461</v>
+        <v>457</v>
       </c>
       <c r="D141" s="4"/>
       <c r="E141" s="4"/>
       <c r="F141" s="4" t="s">
-        <v>462</v>
+        <v>458</v>
       </c>
       <c r="G141" s="4"/>
       <c r="H141" s="4"/>
@@ -10134,18 +10146,18 @@
     </row>
     <row r="142" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A142" s="5" t="s">
-        <v>463</v>
+        <v>459</v>
       </c>
       <c r="B142" s="4" t="s">
-        <v>464</v>
+        <v>460</v>
       </c>
       <c r="C142" s="6" t="s">
-        <v>465</v>
+        <v>461</v>
       </c>
       <c r="D142" s="4"/>
       <c r="E142" s="4"/>
       <c r="F142" s="4" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
       <c r="G142" s="4"/>
       <c r="H142" s="4"/>
@@ -10171,18 +10183,18 @@
     </row>
     <row r="143" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A143" s="5" t="s">
-        <v>467</v>
+        <v>463</v>
       </c>
       <c r="B143" s="4" t="s">
-        <v>468</v>
+        <v>464</v>
       </c>
       <c r="C143" s="6" t="s">
-        <v>469</v>
+        <v>465</v>
       </c>
       <c r="D143" s="4"/>
       <c r="E143" s="4"/>
       <c r="F143" s="4" t="s">
-        <v>470</v>
+        <v>466</v>
       </c>
       <c r="G143" s="4"/>
       <c r="H143" s="4"/>
@@ -10208,18 +10220,18 @@
     </row>
     <row r="144" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A144" s="5" t="s">
-        <v>471</v>
+        <v>467</v>
       </c>
       <c r="B144" s="4" t="s">
-        <v>472</v>
+        <v>468</v>
       </c>
       <c r="C144" s="6" t="s">
-        <v>473</v>
+        <v>469</v>
       </c>
       <c r="D144" s="4"/>
       <c r="E144" s="4"/>
       <c r="F144" s="4" t="s">
-        <v>474</v>
+        <v>470</v>
       </c>
       <c r="G144" s="4"/>
       <c r="H144" s="4"/>
@@ -10245,18 +10257,18 @@
     </row>
     <row r="145" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A145" s="5" t="s">
-        <v>475</v>
+        <v>471</v>
       </c>
       <c r="B145" s="4" t="s">
-        <v>476</v>
+        <v>472</v>
       </c>
       <c r="C145" s="6" t="s">
-        <v>477</v>
+        <v>473</v>
       </c>
       <c r="D145" s="4"/>
       <c r="E145" s="4"/>
       <c r="F145" s="4" t="s">
-        <v>478</v>
+        <v>474</v>
       </c>
       <c r="G145" s="4"/>
       <c r="H145" s="4"/>
@@ -10282,18 +10294,18 @@
     </row>
     <row r="146" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A146" s="5" t="s">
-        <v>479</v>
+        <v>475</v>
       </c>
       <c r="B146" s="4" t="s">
-        <v>480</v>
+        <v>476</v>
       </c>
       <c r="C146" s="6" t="s">
-        <v>481</v>
+        <v>477</v>
       </c>
       <c r="D146" s="4"/>
       <c r="E146" s="4"/>
       <c r="F146" s="4" t="s">
-        <v>482</v>
+        <v>478</v>
       </c>
       <c r="G146" s="4"/>
       <c r="H146" s="4"/>
@@ -10319,18 +10331,18 @@
     </row>
     <row r="147" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A147" s="5" t="s">
-        <v>483</v>
+        <v>479</v>
       </c>
       <c r="B147" s="4" t="s">
-        <v>484</v>
+        <v>480</v>
       </c>
       <c r="C147" s="6" t="s">
-        <v>485</v>
+        <v>481</v>
       </c>
       <c r="D147" s="4"/>
       <c r="E147" s="4"/>
       <c r="F147" s="4" t="s">
-        <v>486</v>
+        <v>482</v>
       </c>
       <c r="G147" s="4"/>
       <c r="H147" s="4"/>
@@ -10356,16 +10368,18 @@
     </row>
     <row r="148" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A148" s="5" t="s">
-        <v>487</v>
+        <v>483</v>
       </c>
       <c r="B148" s="4" t="s">
-        <v>488</v>
-      </c>
-      <c r="C148" s="6"/>
+        <v>484</v>
+      </c>
+      <c r="C148" s="6" t="s">
+        <v>485</v>
+      </c>
       <c r="D148" s="4"/>
       <c r="E148" s="4"/>
       <c r="F148" s="4" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="G148" s="4"/>
       <c r="H148" s="4"/>
@@ -10391,16 +10405,16 @@
     </row>
     <row r="149" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A149" s="5" t="s">
-        <v>490</v>
+        <v>487</v>
       </c>
       <c r="B149" s="4" t="s">
-        <v>491</v>
+        <v>488</v>
       </c>
       <c r="C149" s="6"/>
       <c r="D149" s="4"/>
       <c r="E149" s="4"/>
       <c r="F149" s="4" t="s">
-        <v>492</v>
+        <v>489</v>
       </c>
       <c r="G149" s="4"/>
       <c r="H149" s="4"/>
@@ -10426,16 +10440,16 @@
     </row>
     <row r="150" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A150" s="5" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
       <c r="B150" s="4" t="s">
-        <v>494</v>
+        <v>491</v>
       </c>
       <c r="C150" s="6"/>
       <c r="D150" s="4"/>
       <c r="E150" s="4"/>
       <c r="F150" s="4" t="s">
-        <v>495</v>
+        <v>492</v>
       </c>
       <c r="G150" s="4"/>
       <c r="H150" s="4"/>
@@ -10461,16 +10475,16 @@
     </row>
     <row r="151" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A151" s="5" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="B151" s="4" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
       <c r="C151" s="6"/>
       <c r="D151" s="4"/>
       <c r="E151" s="4"/>
       <c r="F151" s="4" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
       <c r="G151" s="4"/>
       <c r="H151" s="4"/>
@@ -10496,16 +10510,16 @@
     </row>
     <row r="152" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A152" s="5" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
       <c r="B152" s="4" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
       <c r="C152" s="6"/>
       <c r="D152" s="4"/>
       <c r="E152" s="4"/>
       <c r="F152" s="4" t="s">
-        <v>501</v>
+        <v>498</v>
       </c>
       <c r="G152" s="4"/>
       <c r="H152" s="4"/>
@@ -10531,16 +10545,16 @@
     </row>
     <row r="153" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A153" s="5" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
       <c r="B153" s="4" t="s">
-        <v>503</v>
+        <v>500</v>
       </c>
       <c r="C153" s="6"/>
       <c r="D153" s="4"/>
       <c r="E153" s="4"/>
       <c r="F153" s="4" t="s">
-        <v>504</v>
+        <v>501</v>
       </c>
       <c r="G153" s="4"/>
       <c r="H153" s="4"/>
@@ -10566,16 +10580,16 @@
     </row>
     <row r="154" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A154" s="5" t="s">
-        <v>505</v>
+        <v>502</v>
       </c>
       <c r="B154" s="4" t="s">
-        <v>506</v>
+        <v>503</v>
       </c>
       <c r="C154" s="6"/>
       <c r="D154" s="4"/>
       <c r="E154" s="4"/>
       <c r="F154" s="4" t="s">
-        <v>507</v>
+        <v>504</v>
       </c>
       <c r="G154" s="4"/>
       <c r="H154" s="4"/>
@@ -10601,16 +10615,16 @@
     </row>
     <row r="155" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A155" s="5" t="s">
-        <v>508</v>
+        <v>505</v>
       </c>
       <c r="B155" s="4" t="s">
-        <v>509</v>
+        <v>506</v>
       </c>
       <c r="C155" s="6"/>
       <c r="D155" s="4"/>
       <c r="E155" s="4"/>
       <c r="F155" s="4" t="s">
-        <v>510</v>
+        <v>507</v>
       </c>
       <c r="G155" s="4"/>
       <c r="H155" s="4"/>
@@ -10636,16 +10650,16 @@
     </row>
     <row r="156" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A156" s="5" t="s">
-        <v>511</v>
+        <v>508</v>
       </c>
       <c r="B156" s="4" t="s">
-        <v>512</v>
+        <v>509</v>
       </c>
       <c r="C156" s="6"/>
       <c r="D156" s="4"/>
       <c r="E156" s="4"/>
       <c r="F156" s="4" t="s">
-        <v>513</v>
+        <v>510</v>
       </c>
       <c r="G156" s="4"/>
       <c r="H156" s="4"/>
@@ -10670,17 +10684,23 @@
       <c r="AA156" s="2"/>
     </row>
     <row r="157" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A157" s="2"/>
-      <c r="B157" s="2"/>
-      <c r="C157" s="8"/>
-      <c r="D157" s="2"/>
-      <c r="E157" s="2"/>
-      <c r="F157" s="2"/>
-      <c r="G157" s="2"/>
-      <c r="H157" s="2"/>
-      <c r="I157" s="2"/>
-      <c r="J157" s="2"/>
-      <c r="K157" s="2"/>
+      <c r="A157" s="5" t="s">
+        <v>511</v>
+      </c>
+      <c r="B157" s="4" t="s">
+        <v>512</v>
+      </c>
+      <c r="C157" s="6"/>
+      <c r="D157" s="4"/>
+      <c r="E157" s="4"/>
+      <c r="F157" s="4" t="s">
+        <v>513</v>
+      </c>
+      <c r="G157" s="4"/>
+      <c r="H157" s="4"/>
+      <c r="I157" s="4"/>
+      <c r="J157" s="4"/>
+      <c r="K157" s="4"/>
       <c r="L157" s="2"/>
       <c r="M157" s="2"/>
       <c r="N157" s="2"/>
@@ -35203,79 +35223,37 @@
       <c r="Z1002" s="2"/>
       <c r="AA1002" s="2"/>
     </row>
+    <row r="1003" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1003" s="2"/>
+      <c r="B1003" s="2"/>
+      <c r="C1003" s="8"/>
+      <c r="D1003" s="2"/>
+      <c r="E1003" s="2"/>
+      <c r="F1003" s="2"/>
+      <c r="G1003" s="2"/>
+      <c r="H1003" s="2"/>
+      <c r="I1003" s="2"/>
+      <c r="J1003" s="2"/>
+      <c r="K1003" s="2"/>
+      <c r="L1003" s="2"/>
+      <c r="M1003" s="2"/>
+      <c r="N1003" s="2"/>
+      <c r="O1003" s="2"/>
+      <c r="P1003" s="2"/>
+      <c r="Q1003" s="2"/>
+      <c r="R1003" s="2"/>
+      <c r="S1003" s="2"/>
+      <c r="T1003" s="2"/>
+      <c r="U1003" s="2"/>
+      <c r="V1003" s="2"/>
+      <c r="W1003" s="2"/>
+      <c r="X1003" s="2"/>
+      <c r="Y1003" s="2"/>
+      <c r="Z1003" s="2"/>
+      <c r="AA1003" s="2"/>
+    </row>
   </sheetData>
   <mergeCells count="84">
-    <mergeCell ref="H35:H38"/>
-    <mergeCell ref="I35:I38"/>
-    <mergeCell ref="J35:J38"/>
-    <mergeCell ref="A35:A38"/>
-    <mergeCell ref="B35:B38"/>
-    <mergeCell ref="C35:C38"/>
-    <mergeCell ref="D35:D38"/>
-    <mergeCell ref="E35:E38"/>
-    <mergeCell ref="F35:F38"/>
-    <mergeCell ref="G35:G38"/>
-    <mergeCell ref="H45:H71"/>
-    <mergeCell ref="I45:I71"/>
-    <mergeCell ref="J45:J71"/>
-    <mergeCell ref="A45:A71"/>
-    <mergeCell ref="B45:B71"/>
-    <mergeCell ref="C45:C71"/>
-    <mergeCell ref="D45:D71"/>
-    <mergeCell ref="E45:E71"/>
-    <mergeCell ref="F45:F71"/>
-    <mergeCell ref="G45:G71"/>
-    <mergeCell ref="H76:H80"/>
-    <mergeCell ref="I76:I80"/>
-    <mergeCell ref="J76:J80"/>
-    <mergeCell ref="A76:A80"/>
-    <mergeCell ref="B76:B80"/>
-    <mergeCell ref="C76:C80"/>
-    <mergeCell ref="D76:D80"/>
-    <mergeCell ref="E76:E80"/>
-    <mergeCell ref="F76:F80"/>
-    <mergeCell ref="G76:G80"/>
-    <mergeCell ref="H81:H84"/>
-    <mergeCell ref="I81:I84"/>
-    <mergeCell ref="J81:J84"/>
-    <mergeCell ref="A81:A84"/>
-    <mergeCell ref="B81:B84"/>
-    <mergeCell ref="C81:C84"/>
-    <mergeCell ref="D81:D84"/>
-    <mergeCell ref="E81:E84"/>
-    <mergeCell ref="F81:F84"/>
-    <mergeCell ref="G81:G84"/>
-    <mergeCell ref="I1:I3"/>
-    <mergeCell ref="J1:J3"/>
-    <mergeCell ref="K1:K3"/>
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="B1:B3"/>
-    <mergeCell ref="C1:C3"/>
-    <mergeCell ref="D1:D3"/>
-    <mergeCell ref="E1:E3"/>
-    <mergeCell ref="G1:G3"/>
-    <mergeCell ref="H1:H3"/>
-    <mergeCell ref="H16:H17"/>
-    <mergeCell ref="I16:I17"/>
-    <mergeCell ref="J16:J17"/>
-    <mergeCell ref="A16:A17"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="D16:D17"/>
-    <mergeCell ref="E16:E17"/>
-    <mergeCell ref="F16:F17"/>
-    <mergeCell ref="G16:G17"/>
-    <mergeCell ref="H20:H21"/>
-    <mergeCell ref="I20:I21"/>
-    <mergeCell ref="J20:J21"/>
-    <mergeCell ref="K20:K21"/>
-    <mergeCell ref="A20:A21"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="C20:C21"/>
-    <mergeCell ref="D20:D21"/>
-    <mergeCell ref="E20:E21"/>
-    <mergeCell ref="F20:F21"/>
-    <mergeCell ref="G20:G21"/>
     <mergeCell ref="J119:J120"/>
     <mergeCell ref="A85:A88"/>
     <mergeCell ref="B85:B88"/>
@@ -35289,6 +35267,77 @@
     <mergeCell ref="G119:G120"/>
     <mergeCell ref="H119:H120"/>
     <mergeCell ref="I119:I120"/>
+    <mergeCell ref="H20:H21"/>
+    <mergeCell ref="I20:I21"/>
+    <mergeCell ref="J20:J21"/>
+    <mergeCell ref="K20:K21"/>
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="C20:C21"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="E20:E21"/>
+    <mergeCell ref="F20:F21"/>
+    <mergeCell ref="G20:G21"/>
+    <mergeCell ref="H16:H17"/>
+    <mergeCell ref="I16:I17"/>
+    <mergeCell ref="J16:J17"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="D16:D17"/>
+    <mergeCell ref="E16:E17"/>
+    <mergeCell ref="F16:F17"/>
+    <mergeCell ref="G16:G17"/>
+    <mergeCell ref="I1:I3"/>
+    <mergeCell ref="J1:J3"/>
+    <mergeCell ref="K1:K3"/>
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="B1:B3"/>
+    <mergeCell ref="C1:C3"/>
+    <mergeCell ref="D1:D3"/>
+    <mergeCell ref="E1:E3"/>
+    <mergeCell ref="G1:G3"/>
+    <mergeCell ref="H1:H3"/>
+    <mergeCell ref="H81:H84"/>
+    <mergeCell ref="I81:I84"/>
+    <mergeCell ref="J81:J84"/>
+    <mergeCell ref="A81:A84"/>
+    <mergeCell ref="B81:B84"/>
+    <mergeCell ref="C81:C84"/>
+    <mergeCell ref="D81:D84"/>
+    <mergeCell ref="E81:E84"/>
+    <mergeCell ref="F81:F84"/>
+    <mergeCell ref="G81:G84"/>
+    <mergeCell ref="H76:H80"/>
+    <mergeCell ref="I76:I80"/>
+    <mergeCell ref="J76:J80"/>
+    <mergeCell ref="A76:A80"/>
+    <mergeCell ref="B76:B80"/>
+    <mergeCell ref="C76:C80"/>
+    <mergeCell ref="D76:D80"/>
+    <mergeCell ref="E76:E80"/>
+    <mergeCell ref="F76:F80"/>
+    <mergeCell ref="G76:G80"/>
+    <mergeCell ref="H45:H71"/>
+    <mergeCell ref="I45:I71"/>
+    <mergeCell ref="J45:J71"/>
+    <mergeCell ref="A45:A71"/>
+    <mergeCell ref="B45:B71"/>
+    <mergeCell ref="C45:C71"/>
+    <mergeCell ref="D45:D71"/>
+    <mergeCell ref="E45:E71"/>
+    <mergeCell ref="F45:F71"/>
+    <mergeCell ref="G45:G71"/>
+    <mergeCell ref="H35:H38"/>
+    <mergeCell ref="I35:I38"/>
+    <mergeCell ref="J35:J38"/>
+    <mergeCell ref="A35:A38"/>
+    <mergeCell ref="B35:B38"/>
+    <mergeCell ref="C35:C38"/>
+    <mergeCell ref="D35:D38"/>
+    <mergeCell ref="E35:E38"/>
+    <mergeCell ref="F35:F38"/>
+    <mergeCell ref="G35:G38"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="portrait"/>

</xml_diff>